<commit_message>
sc8505 & sc85853 update
</commit_message>
<xml_diff>
--- a/misc/regmap/sc8563_1p1_regmap.xlsx
+++ b/misc/regmap/sc8563_1p1_regmap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\labmachine\south_git\misc\regmap\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lab_Experiement\south_lab\misc\regmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2AA1596A-6D05-4FBB-8AC6-905B5C88A2D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2B8036-AC80-4ECA-81CB-D23A57569A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38295" yWindow="2310" windowWidth="29340" windowHeight="20985" xr2:uid="{04341A28-7F9A-4CCC-96B6-6759C0F557E5}"/>
+    <workbookView xWindow="696" yWindow="2244" windowWidth="22416" windowHeight="12696" xr2:uid="{04341A28-7F9A-4CCC-96B6-6759C0F557E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -738,10 +738,6 @@
     <t>VOUT_TH_CHG_EN_FLAG</t>
   </si>
   <si>
-    <t>DEVICE_VER]7:0]</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>VEXT1_REMOVE_FLAG</t>
   </si>
   <si>
@@ -1266,6 +1262,9 @@
   <si>
     <t>RW</t>
     <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DEVICE_VER[7:0]</t>
   </si>
 </sst>
 </file>
@@ -1276,7 +1275,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1284,13 +1283,13 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1298,7 +1297,7 @@
     <font>
       <sz val="8"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Aptos Narrow"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -1375,9 +1374,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
     </xf>
@@ -1387,6 +1383,9 @@
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1395,466 +1394,10 @@
     </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="표준 2" xfId="1" xr:uid="{2F0B188C-9CDA-490A-9027-6F91E456A318}"/>
   </cellStyles>
-  <dxfs count="65">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor indexed="10"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -2185,25 +1728,25 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D53D8F-E1AB-4E17-A001-E0EB1C0ED563}">
   <dimension ref="A1:M246"/>
-  <sheetFormatPr defaultRowHeight="10.8" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="9.6" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="6.8984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.3984375" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="5.69921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="4.09765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.09765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="20.59765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="19.296875" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="18.09765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="20.69921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="22" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.09765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="20.09765625" style="3" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="23.69921875" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="16384" width="8.796875" style="3"/>
+    <col min="1" max="1" width="6.8984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.3984375" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="5.69921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="4.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="5.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="20.59765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="19.296875" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="20.69921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.09765625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="23.69921875" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="16384" width="8.796875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2219,18 +1762,18 @@
       <c r="E1" s="1" t="s">
         <v>217</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-    </row>
-    <row r="2" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F1" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="5"/>
+      <c r="K1" s="5"/>
+      <c r="L1" s="5"/>
+      <c r="M1" s="5"/>
+    </row>
+    <row r="2" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -2271,7 +1814,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -2288,31 +1831,31 @@
         <v>218</v>
       </c>
       <c r="F3" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="G3" s="1" t="s">
         <v>227</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="H3" s="1" t="s">
         <v>228</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="I3" s="1" t="s">
         <v>229</v>
       </c>
-      <c r="I3" s="1" t="s">
+      <c r="J3" s="1" t="s">
         <v>230</v>
       </c>
-      <c r="J3" s="1" t="s">
+      <c r="K3" s="1" t="s">
         <v>231</v>
       </c>
-      <c r="K3" s="1" t="s">
+      <c r="L3" s="1" t="s">
         <v>232</v>
       </c>
-      <c r="L3" s="1" t="s">
+      <c r="M3" s="1" t="s">
         <v>233</v>
       </c>
-      <c r="M3" s="1" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="4" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -2329,31 +1872,31 @@
         <v>218</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>198</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I4" s="1" t="s">
         <v>199</v>
       </c>
       <c r="J4" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="K4" s="1" t="s">
         <v>237</v>
       </c>
-      <c r="K4" s="1" t="s">
+      <c r="L4" s="1" t="s">
         <v>238</v>
-      </c>
-      <c r="L4" s="1" t="s">
-        <v>239</v>
       </c>
       <c r="M4" s="1" t="s">
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -2370,13 +1913,13 @@
         <v>218</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>201</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="I5" s="1" t="s">
         <v>84</v>
@@ -2385,16 +1928,16 @@
         <v>85</v>
       </c>
       <c r="K5" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="L5" s="1" t="s">
         <v>242</v>
       </c>
-      <c r="L5" s="1" t="s">
+      <c r="M5" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="M5" s="1" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="6" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>10</v>
       </c>
@@ -2411,31 +1954,31 @@
         <v>218</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>245</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="H6" s="1" t="s">
         <v>246</v>
       </c>
-      <c r="H6" s="1" t="s">
+      <c r="I6" s="1" t="s">
         <v>247</v>
       </c>
-      <c r="I6" s="1" t="s">
+      <c r="J6" s="1" t="s">
         <v>248</v>
       </c>
-      <c r="J6" s="1" t="s">
+      <c r="K6" s="1" t="s">
         <v>249</v>
       </c>
-      <c r="K6" s="1" t="s">
+      <c r="L6" s="1" t="s">
         <v>250</v>
       </c>
-      <c r="L6" s="1" t="s">
+      <c r="M6" s="1" t="s">
         <v>251</v>
       </c>
-      <c r="M6" s="1" t="s">
-        <v>252</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
@@ -2452,22 +1995,22 @@
         <v>218</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>253</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="H7" s="1" t="s">
         <v>254</v>
       </c>
-      <c r="H7" s="1" t="s">
+      <c r="I7" s="1" t="s">
         <v>255</v>
       </c>
-      <c r="I7" s="1" t="s">
+      <c r="J7" s="1" t="s">
         <v>256</v>
       </c>
-      <c r="J7" s="1" t="s">
+      <c r="K7" s="1" t="s">
         <v>257</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>258</v>
       </c>
       <c r="L7" s="1" t="s">
         <v>202</v>
@@ -2476,7 +2019,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>12</v>
       </c>
@@ -2487,37 +2030,37 @@
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F8" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="G8" s="1" t="s">
         <v>259</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="H8" s="1" t="s">
         <v>260</v>
       </c>
-      <c r="H8" s="1" t="s">
+      <c r="I8" s="1" t="s">
         <v>261</v>
-      </c>
-      <c r="I8" s="1" t="s">
-        <v>262</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>86</v>
       </c>
       <c r="K8" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="L8" s="1" t="s">
         <v>263</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>264</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -2528,37 +2071,37 @@
         <v>1</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F9" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="G9" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="H9" s="1" t="s">
         <v>266</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="I9" s="1" t="s">
         <v>267</v>
       </c>
-      <c r="I9" s="1" t="s">
+      <c r="J9" s="1" t="s">
         <v>268</v>
       </c>
-      <c r="J9" s="1" t="s">
+      <c r="K9" s="1" t="s">
         <v>269</v>
       </c>
-      <c r="K9" s="1" t="s">
+      <c r="L9" s="1" t="s">
         <v>270</v>
       </c>
-      <c r="L9" s="1" t="s">
+      <c r="M9" s="1" t="s">
         <v>271</v>
       </c>
-      <c r="M9" s="1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="10" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>14</v>
       </c>
@@ -2569,37 +2112,37 @@
         <v>1</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>88</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I10" s="1" t="s">
         <v>90</v>
       </c>
       <c r="J10" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="K10" s="1" t="s">
         <v>274</v>
       </c>
-      <c r="K10" s="1" t="s">
+      <c r="L10" s="1" t="s">
         <v>275</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>276</v>
       </c>
       <c r="M10" s="1" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>52</v>
       </c>
@@ -2610,19 +2153,19 @@
         <v>1</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>92</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="I11" s="1" t="s">
         <v>93</v>
@@ -2631,16 +2174,16 @@
         <v>94</v>
       </c>
       <c r="K11" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="L11" s="1" t="s">
         <v>279</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="M11" s="1" t="s">
         <v>280</v>
       </c>
-      <c r="M11" s="1" t="s">
-        <v>281</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="12" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>54</v>
       </c>
@@ -2651,37 +2194,37 @@
         <v>1</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F12" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="G12" s="1" t="s">
         <v>282</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="H12" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="H12" s="1" t="s">
+      <c r="I12" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="I12" s="1" t="s">
+      <c r="J12" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="J12" s="1" t="s">
+      <c r="K12" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="K12" s="1" t="s">
+      <c r="L12" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="L12" s="1" t="s">
+      <c r="M12" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="M12" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="13" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>55</v>
       </c>
@@ -2692,28 +2235,28 @@
         <v>1</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F13" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="G13" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="H13" s="1" t="s">
         <v>291</v>
       </c>
-      <c r="H13" s="1" t="s">
+      <c r="I13" s="1" t="s">
         <v>292</v>
       </c>
-      <c r="I13" s="1" t="s">
+      <c r="J13" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="J13" s="1" t="s">
+      <c r="K13" s="1" t="s">
         <v>294</v>
-      </c>
-      <c r="K13" s="1" t="s">
-        <v>295</v>
       </c>
       <c r="L13" s="1" t="s">
         <v>95</v>
@@ -2722,7 +2265,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>57</v>
       </c>
@@ -2739,31 +2282,31 @@
         <v>218</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G14" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="H14" s="1" t="s">
         <v>296</v>
       </c>
-      <c r="H14" s="1" t="s">
+      <c r="I14" s="1" t="s">
         <v>297</v>
-      </c>
-      <c r="I14" s="1" t="s">
-        <v>298</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>203</v>
       </c>
       <c r="K14" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="L14" s="1" t="s">
         <v>299</v>
-      </c>
-      <c r="L14" s="1" t="s">
-        <v>300</v>
       </c>
       <c r="M14" s="1" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>58</v>
       </c>
@@ -2780,31 +2323,31 @@
         <v>218</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="H15" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="I15" s="1" t="s">
         <v>301</v>
       </c>
-      <c r="I15" s="1" t="s">
+      <c r="J15" s="1" t="s">
         <v>302</v>
       </c>
-      <c r="J15" s="1" t="s">
+      <c r="K15" s="1" t="s">
         <v>303</v>
       </c>
-      <c r="K15" s="1" t="s">
+      <c r="L15" s="1" t="s">
         <v>304</v>
       </c>
-      <c r="L15" s="1" t="s">
+      <c r="M15" s="1" t="s">
         <v>305</v>
       </c>
-      <c r="M15" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="16" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>59</v>
       </c>
@@ -2821,31 +2364,31 @@
         <v>218</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>206</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J16" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="K16" s="1" t="s">
         <v>309</v>
       </c>
-      <c r="K16" s="1" t="s">
+      <c r="L16" s="1" t="s">
         <v>310</v>
-      </c>
-      <c r="L16" s="1" t="s">
-        <v>311</v>
       </c>
       <c r="M16" s="1" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2862,13 +2405,13 @@
         <v>218</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G17" s="1" t="s">
         <v>208</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="I17" s="1" t="s">
         <v>96</v>
@@ -2877,16 +2420,16 @@
         <v>97</v>
       </c>
       <c r="K17" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="L17" s="1" t="s">
         <v>314</v>
       </c>
-      <c r="L17" s="1" t="s">
+      <c r="M17" s="1" t="s">
         <v>315</v>
       </c>
-      <c r="M17" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="18" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2903,31 +2446,31 @@
         <v>218</v>
       </c>
       <c r="F18" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="G18" s="1" t="s">
         <v>317</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="H18" s="1" t="s">
         <v>318</v>
       </c>
-      <c r="H18" s="1" t="s">
+      <c r="I18" s="1" t="s">
         <v>319</v>
       </c>
-      <c r="I18" s="1" t="s">
+      <c r="J18" s="1" t="s">
         <v>320</v>
       </c>
-      <c r="J18" s="1" t="s">
+      <c r="K18" s="1" t="s">
         <v>321</v>
       </c>
-      <c r="K18" s="1" t="s">
+      <c r="L18" s="1" t="s">
         <v>322</v>
       </c>
-      <c r="L18" s="1" t="s">
+      <c r="M18" s="1" t="s">
         <v>323</v>
       </c>
-      <c r="M18" s="1" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="19" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2944,22 +2487,22 @@
         <v>218</v>
       </c>
       <c r="F19" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="G19" s="1" t="s">
         <v>325</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="H19" s="1" t="s">
         <v>326</v>
       </c>
-      <c r="H19" s="1" t="s">
+      <c r="I19" s="1" t="s">
         <v>327</v>
       </c>
-      <c r="I19" s="1" t="s">
+      <c r="J19" s="1" t="s">
         <v>328</v>
       </c>
-      <c r="J19" s="1" t="s">
+      <c r="K19" s="1" t="s">
         <v>329</v>
-      </c>
-      <c r="K19" s="1" t="s">
-        <v>330</v>
       </c>
       <c r="L19" s="1" t="s">
         <v>209</v>
@@ -2968,7 +2511,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2979,31 +2522,31 @@
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F20" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="G20" s="1" t="s">
         <v>331</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="H20" s="5" t="s">
         <v>332</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="I20" s="5"/>
+      <c r="J20" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="K20" s="5" t="s">
         <v>333</v>
       </c>
-      <c r="I20" s="2"/>
-      <c r="J20" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="K20" s="2" t="s">
-        <v>334</v>
-      </c>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
-    </row>
-    <row r="21" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="L20" s="5"/>
+      <c r="M20" s="5"/>
+    </row>
+    <row r="21" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -3014,7 +2557,7 @@
         <v>1</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E21" s="1" t="s">
         <v>218</v>
@@ -3023,24 +2566,24 @@
         <v>104</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>335</v>
-      </c>
-      <c r="I21" s="2"/>
+        <v>235</v>
+      </c>
+      <c r="H21" s="5" t="s">
+        <v>334</v>
+      </c>
+      <c r="I21" s="5"/>
       <c r="J21" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="K21" s="2" t="s">
-        <v>336</v>
-      </c>
-      <c r="L21" s="2"/>
+      <c r="K21" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="L21" s="5"/>
       <c r="M21" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -3051,29 +2594,29 @@
         <v>1</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E22" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="H22" s="2" t="s">
+        <v>235</v>
+      </c>
+      <c r="H22" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="I22" s="5"/>
+      <c r="J22" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2" t="s">
-        <v>338</v>
-      </c>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K22" s="5"/>
+      <c r="L22" s="5"/>
+      <c r="M22" s="5"/>
+    </row>
+    <row r="23" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -3084,7 +2627,7 @@
         <v>1</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E23" s="1" t="s">
         <v>218</v>
@@ -3095,10 +2638,10 @@
       <c r="G23" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="H23" s="2" t="s">
-        <v>339</v>
-      </c>
-      <c r="I23" s="2"/>
+      <c r="H23" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="I23" s="5"/>
       <c r="J23" s="1" t="s">
         <v>102</v>
       </c>
@@ -3112,7 +2655,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -3123,7 +2666,7 @@
         <v>1</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E24" s="1" t="s">
         <v>218</v>
@@ -3146,12 +2689,12 @@
       <c r="K24" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="L24" s="2" t="s">
+      <c r="L24" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="M24" s="2"/>
-    </row>
-    <row r="25" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="M24" s="5"/>
+    </row>
+    <row r="25" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -3162,33 +2705,33 @@
         <v>1</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E25" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F25" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="G25" s="1" t="s">
         <v>340</v>
       </c>
-      <c r="G25" s="1" t="s">
+      <c r="H25" s="1" t="s">
         <v>341</v>
       </c>
-      <c r="H25" s="1" t="s">
+      <c r="I25" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="I25" s="1" t="s">
+      <c r="J25" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="K25" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="J25" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="K25" s="2" t="s">
-        <v>344</v>
-      </c>
-      <c r="L25" s="2"/>
-      <c r="M25" s="2"/>
-    </row>
-    <row r="26" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+    </row>
+    <row r="26" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -3199,33 +2742,33 @@
         <v>1</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E26" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F26" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="G26" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="G26" s="1" t="s">
+      <c r="H26" s="1" t="s">
         <v>346</v>
       </c>
-      <c r="H26" s="1" t="s">
+      <c r="I26" s="1" t="s">
         <v>347</v>
       </c>
-      <c r="I26" s="1" t="s">
+      <c r="J26" s="1" t="s">
         <v>348</v>
       </c>
-      <c r="J26" s="1" t="s">
+      <c r="K26" s="5" t="s">
         <v>349</v>
       </c>
-      <c r="K26" s="2" t="s">
-        <v>350</v>
-      </c>
-      <c r="L26" s="2"/>
-      <c r="M26" s="2"/>
-    </row>
-    <row r="27" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="L26" s="5"/>
+      <c r="M26" s="5"/>
+    </row>
+    <row r="27" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>66</v>
       </c>
@@ -3236,22 +2779,22 @@
         <v>1</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E27" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F27" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G27" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>352</v>
-      </c>
       <c r="H27" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="J27" s="1" t="s">
         <v>112</v>
@@ -3259,12 +2802,12 @@
       <c r="K27" s="1" t="s">
         <v>113</v>
       </c>
-      <c r="L27" s="2" t="s">
+      <c r="L27" s="5" t="s">
         <v>135</v>
       </c>
-      <c r="M27" s="2"/>
-    </row>
-    <row r="28" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="M27" s="5"/>
+    </row>
+    <row r="28" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>68</v>
       </c>
@@ -3275,23 +2818,23 @@
         <v>1</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E28" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F28" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="G28" s="2"/>
-      <c r="H28" s="2"/>
-      <c r="I28" s="2"/>
-      <c r="J28" s="2"/>
-      <c r="K28" s="2"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="2"/>
-    </row>
-    <row r="29" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F28" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="G28" s="5"/>
+      <c r="H28" s="5"/>
+      <c r="I28" s="5"/>
+      <c r="J28" s="5"/>
+      <c r="K28" s="5"/>
+      <c r="L28" s="5"/>
+      <c r="M28" s="5"/>
+    </row>
+    <row r="29" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>70</v>
       </c>
@@ -3302,23 +2845,23 @@
         <v>1</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E29" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F29" s="2" t="s">
-        <v>354</v>
-      </c>
-      <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
-      <c r="K29" s="2"/>
-      <c r="L29" s="2"/>
-      <c r="M29" s="2"/>
-    </row>
-    <row r="30" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F29" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="G29" s="5"/>
+      <c r="H29" s="5"/>
+      <c r="I29" s="5"/>
+      <c r="J29" s="5"/>
+      <c r="K29" s="5"/>
+      <c r="L29" s="5"/>
+      <c r="M29" s="5"/>
+    </row>
+    <row r="30" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>72</v>
       </c>
@@ -3329,25 +2872,25 @@
         <v>1</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E30" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F30" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="G30" s="5" t="s">
         <v>355</v>
       </c>
-      <c r="G30" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="H30" s="2"/>
-      <c r="I30" s="2"/>
-      <c r="J30" s="2"/>
-      <c r="K30" s="2"/>
-      <c r="L30" s="2"/>
-      <c r="M30" s="2"/>
-    </row>
-    <row r="31" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="H30" s="5"/>
+      <c r="I30" s="5"/>
+      <c r="J30" s="5"/>
+      <c r="K30" s="5"/>
+      <c r="L30" s="5"/>
+      <c r="M30" s="5"/>
+    </row>
+    <row r="31" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>74</v>
       </c>
@@ -3358,7 +2901,7 @@
         <v>1</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E31" s="1" t="s">
         <v>218</v>
@@ -3370,7 +2913,7 @@
         <v>115</v>
       </c>
       <c r="H31" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="I31" s="1" t="s">
         <v>116</v>
@@ -3381,12 +2924,12 @@
       <c r="K31" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="L31" s="2" t="s">
+      <c r="L31" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="M31" s="2"/>
-    </row>
-    <row r="32" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="M31" s="5"/>
+    </row>
+    <row r="32" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>76</v>
       </c>
@@ -3397,23 +2940,23 @@
         <v>1</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E32" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F32" s="2" t="s">
-        <v>357</v>
-      </c>
-      <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="2"/>
-      <c r="K32" s="2"/>
-      <c r="L32" s="2"/>
-      <c r="M32" s="2"/>
-    </row>
-    <row r="33" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F32" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="G32" s="5"/>
+      <c r="H32" s="5"/>
+      <c r="I32" s="5"/>
+      <c r="J32" s="5"/>
+      <c r="K32" s="5"/>
+      <c r="L32" s="5"/>
+      <c r="M32" s="5"/>
+    </row>
+    <row r="33" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>25</v>
       </c>
@@ -3424,25 +2967,25 @@
         <v>1</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E33" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>356</v>
-      </c>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-    </row>
-    <row r="34" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+        <v>357</v>
+      </c>
+      <c r="G33" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="H33" s="5"/>
+      <c r="I33" s="5"/>
+      <c r="J33" s="5"/>
+      <c r="K33" s="5"/>
+      <c r="L33" s="5"/>
+      <c r="M33" s="5"/>
+    </row>
+    <row r="34" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>26</v>
       </c>
@@ -3453,31 +2996,31 @@
         <v>1</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E34" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F34" s="4" t="s">
+      <c r="F34" s="3" t="s">
         <v>119</v>
       </c>
-      <c r="G34" s="2" t="s">
+      <c r="G34" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="H34" s="5"/>
+      <c r="I34" s="5"/>
+      <c r="J34" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="L34" s="5" t="s">
         <v>359</v>
       </c>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="K34" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="L34" s="2" t="s">
-        <v>360</v>
-      </c>
-      <c r="M34" s="2"/>
-    </row>
-    <row r="35" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="M34" s="5"/>
+    </row>
+    <row r="35" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>27</v>
       </c>
@@ -3488,23 +3031,23 @@
         <v>1</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E35" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F35" s="2" t="s">
-        <v>361</v>
-      </c>
-      <c r="G35" s="2"/>
-      <c r="H35" s="2"/>
-      <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-    </row>
-    <row r="36" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F35" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="G35" s="5"/>
+      <c r="H35" s="5"/>
+      <c r="I35" s="5"/>
+      <c r="J35" s="5"/>
+      <c r="K35" s="5"/>
+      <c r="L35" s="5"/>
+      <c r="M35" s="5"/>
+    </row>
+    <row r="36" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>28</v>
       </c>
@@ -3515,29 +3058,29 @@
         <v>1</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E36" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F36" s="4" t="s">
+      <c r="F36" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="G36" s="2" t="s">
+      <c r="G36" s="5" t="s">
+        <v>361</v>
+      </c>
+      <c r="H36" s="5"/>
+      <c r="I36" s="5" t="s">
         <v>362</v>
       </c>
-      <c r="H36" s="2"/>
-      <c r="I36" s="2" t="s">
+      <c r="J36" s="5"/>
+      <c r="K36" s="5" t="s">
         <v>363</v>
       </c>
-      <c r="J36" s="2"/>
-      <c r="K36" s="2" t="s">
-        <v>364</v>
-      </c>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-    </row>
-    <row r="37" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="L36" s="5"/>
+      <c r="M36" s="5"/>
+    </row>
+    <row r="37" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>29</v>
       </c>
@@ -3548,29 +3091,29 @@
         <v>1</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E37" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F37" s="3" t="s">
+        <v>364</v>
+      </c>
+      <c r="G37" s="5" t="s">
         <v>365</v>
       </c>
-      <c r="G37" s="2" t="s">
+      <c r="H37" s="5"/>
+      <c r="I37" s="5" t="s">
         <v>366</v>
       </c>
-      <c r="H37" s="2"/>
-      <c r="I37" s="2" t="s">
+      <c r="J37" s="5"/>
+      <c r="K37" s="5" t="s">
         <v>367</v>
       </c>
-      <c r="J37" s="2"/>
-      <c r="K37" s="2" t="s">
-        <v>368</v>
-      </c>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-    </row>
-    <row r="38" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="L37" s="5"/>
+      <c r="M37" s="5"/>
+    </row>
+    <row r="38" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>30</v>
       </c>
@@ -3581,27 +3124,27 @@
         <v>1</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E38" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F38" s="4" t="s">
+      <c r="F38" s="3" t="s">
         <v>123</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H38" s="2" t="s">
-        <v>369</v>
-      </c>
-      <c r="I38" s="2"/>
-      <c r="J38" s="2"/>
-      <c r="K38" s="2"/>
-      <c r="L38" s="2"/>
-      <c r="M38" s="2"/>
-    </row>
-    <row r="39" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G38" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="I38" s="5"/>
+      <c r="J38" s="5"/>
+      <c r="K38" s="5"/>
+      <c r="L38" s="5"/>
+      <c r="M38" s="5"/>
+    </row>
+    <row r="39" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>31</v>
       </c>
@@ -3612,7 +3155,7 @@
         <v>1</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E39" s="1" t="s">
         <v>218</v>
@@ -3626,23 +3169,23 @@
       <c r="H39" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="I39" s="4" t="s">
+      <c r="I39" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="J39" s="4" t="s">
+      <c r="J39" s="3" t="s">
         <v>128</v>
       </c>
-      <c r="K39" s="4" t="s">
+      <c r="K39" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="L39" s="4" t="s">
+      <c r="L39" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="M39" s="4" t="s">
+      <c r="M39" s="3" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>32</v>
       </c>
@@ -3653,31 +3196,31 @@
         <v>1</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E40" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F40" s="2" t="s">
+      <c r="F40" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="G40" s="5"/>
+      <c r="H40" s="5" t="s">
         <v>370</v>
       </c>
-      <c r="G40" s="2"/>
-      <c r="H40" s="2" t="s">
+      <c r="I40" s="5"/>
+      <c r="J40" s="5" t="s">
         <v>371</v>
       </c>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2" t="s">
-        <v>372</v>
-      </c>
-      <c r="K40" s="2"/>
-      <c r="L40" s="4" t="s">
+      <c r="K40" s="5"/>
+      <c r="L40" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="M40" s="4" t="s">
+      <c r="M40" s="3" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>33</v>
       </c>
@@ -3688,31 +3231,31 @@
         <v>1</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E41" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F41" s="2" t="s">
+      <c r="F41" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5" t="s">
         <v>375</v>
       </c>
-      <c r="G41" s="2"/>
-      <c r="H41" s="2" t="s">
+      <c r="I41" s="5"/>
+      <c r="J41" s="5" t="s">
         <v>376</v>
       </c>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2" t="s">
-        <v>377</v>
-      </c>
-      <c r="K41" s="2"/>
-      <c r="L41" s="4" t="s">
+      <c r="K41" s="5"/>
+      <c r="L41" s="3" t="s">
+        <v>372</v>
+      </c>
+      <c r="M41" s="3" t="s">
         <v>373</v>
       </c>
-      <c r="M41" s="4" t="s">
-        <v>374</v>
-      </c>
-    </row>
-    <row r="42" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    </row>
+    <row r="42" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>34</v>
       </c>
@@ -3723,37 +3266,37 @@
         <v>1</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E42" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F42" s="4" t="s">
+      <c r="F42" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="G42" s="4" t="s">
+      <c r="G42" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="H42" s="4" t="s">
+      <c r="H42" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="I42" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="K42" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="L42" s="4" t="s">
+      <c r="I42" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J42" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K42" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="L42" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="M42" s="4" t="s">
+      <c r="M42" s="3" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>144</v>
       </c>
@@ -3764,37 +3307,37 @@
         <v>1</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
       <c r="E43" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F43" s="4" t="s">
+      <c r="F43" s="3" t="s">
+        <v>382</v>
+      </c>
+      <c r="G43" s="3" t="s">
         <v>383</v>
       </c>
-      <c r="G43" s="4" t="s">
-        <v>384</v>
-      </c>
-      <c r="H43" s="4" t="s">
+      <c r="H43" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="I43" s="4" t="s">
+      <c r="I43" s="3" t="s">
         <v>177</v>
       </c>
-      <c r="J43" s="4" t="s">
+      <c r="J43" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="K43" s="4" t="s">
+      <c r="K43" s="3" t="s">
         <v>179</v>
       </c>
-      <c r="L43" s="4" t="s">
+      <c r="L43" s="3" t="s">
         <v>180</v>
       </c>
-      <c r="M43" s="4" t="s">
+      <c r="M43" s="3" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>146</v>
       </c>
@@ -3810,26 +3353,26 @@
       <c r="E44" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F44" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I44" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J44" s="2" t="s">
+      <c r="F44" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G44" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H44" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I44" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J44" s="5" t="s">
         <v>190</v>
       </c>
-      <c r="K44" s="2"/>
-      <c r="L44" s="2"/>
-      <c r="M44" s="2"/>
-    </row>
-    <row r="45" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K44" s="5"/>
+      <c r="L44" s="5"/>
+      <c r="M44" s="5"/>
+    </row>
+    <row r="45" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>148</v>
       </c>
@@ -3845,18 +3388,18 @@
       <c r="E45" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F45" s="2" t="s">
+      <c r="F45" s="5" t="s">
         <v>182</v>
       </c>
-      <c r="G45" s="2"/>
-      <c r="H45" s="2"/>
-      <c r="I45" s="2"/>
-      <c r="J45" s="2"/>
-      <c r="K45" s="2"/>
-      <c r="L45" s="2"/>
-      <c r="M45" s="2"/>
-    </row>
-    <row r="46" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G45" s="5"/>
+      <c r="H45" s="5"/>
+      <c r="I45" s="5"/>
+      <c r="J45" s="5"/>
+      <c r="K45" s="5"/>
+      <c r="L45" s="5"/>
+      <c r="M45" s="5"/>
+    </row>
+    <row r="46" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>150</v>
       </c>
@@ -3872,31 +3415,31 @@
       <c r="E46" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F46" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H46" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I46" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J46" s="2" t="s">
+      <c r="F46" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G46" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H46" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I46" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J46" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="K46" s="2"/>
-      <c r="L46" s="2"/>
-      <c r="M46" s="2"/>
-    </row>
-    <row r="47" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K46" s="5"/>
+      <c r="L46" s="5"/>
+      <c r="M46" s="5"/>
+    </row>
+    <row r="47" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>1</v>
@@ -3907,23 +3450,23 @@
       <c r="E47" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F47" s="2" t="s">
+      <c r="F47" s="5" t="s">
         <v>183</v>
       </c>
-      <c r="G47" s="2"/>
-      <c r="H47" s="2"/>
-      <c r="I47" s="2"/>
-      <c r="J47" s="2"/>
-      <c r="K47" s="2"/>
-      <c r="L47" s="2"/>
-      <c r="M47" s="2"/>
-    </row>
-    <row r="48" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G47" s="5"/>
+      <c r="H47" s="5"/>
+      <c r="I47" s="5"/>
+      <c r="J47" s="5"/>
+      <c r="K47" s="5"/>
+      <c r="L47" s="5"/>
+      <c r="M47" s="5"/>
+    </row>
+    <row r="48" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>1</v>
@@ -3934,31 +3477,31 @@
       <c r="E48" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F48" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H48" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I48" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J48" s="2" t="s">
-        <v>385</v>
-      </c>
-      <c r="K48" s="2"/>
-      <c r="L48" s="2"/>
-      <c r="M48" s="2"/>
-    </row>
-    <row r="49" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F48" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G48" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H48" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I48" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J48" s="5" t="s">
+        <v>384</v>
+      </c>
+      <c r="K48" s="5"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="5"/>
+    </row>
+    <row r="49" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>1</v>
@@ -3969,23 +3512,23 @@
       <c r="E49" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F49" s="2" t="s">
-        <v>386</v>
-      </c>
-      <c r="G49" s="2"/>
-      <c r="H49" s="2"/>
-      <c r="I49" s="2"/>
-      <c r="J49" s="2"/>
-      <c r="K49" s="2"/>
-      <c r="L49" s="2"/>
-      <c r="M49" s="2"/>
-    </row>
-    <row r="50" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F49" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="G49" s="5"/>
+      <c r="H49" s="5"/>
+      <c r="I49" s="5"/>
+      <c r="J49" s="5"/>
+      <c r="K49" s="5"/>
+      <c r="L49" s="5"/>
+      <c r="M49" s="5"/>
+    </row>
+    <row r="50" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>1</v>
@@ -3996,31 +3539,31 @@
       <c r="E50" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F50" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H50" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I50" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J50" s="2" t="s">
-        <v>387</v>
-      </c>
-      <c r="K50" s="2"/>
-      <c r="L50" s="2"/>
-      <c r="M50" s="2"/>
-    </row>
-    <row r="51" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F50" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G50" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H50" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I50" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J50" s="5" t="s">
+        <v>386</v>
+      </c>
+      <c r="K50" s="5"/>
+      <c r="L50" s="5"/>
+      <c r="M50" s="5"/>
+    </row>
+    <row r="51" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>1</v>
@@ -4031,18 +3574,18 @@
       <c r="E51" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F51" s="2" t="s">
-        <v>388</v>
-      </c>
-      <c r="G51" s="2"/>
-      <c r="H51" s="2"/>
-      <c r="I51" s="2"/>
-      <c r="J51" s="2"/>
-      <c r="K51" s="2"/>
-      <c r="L51" s="2"/>
-      <c r="M51" s="2"/>
-    </row>
-    <row r="52" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="F51" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="G51" s="5"/>
+      <c r="H51" s="5"/>
+      <c r="I51" s="5"/>
+      <c r="J51" s="5"/>
+      <c r="K51" s="5"/>
+      <c r="L51" s="5"/>
+      <c r="M51" s="5"/>
+    </row>
+    <row r="52" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>38</v>
       </c>
@@ -4058,26 +3601,26 @@
       <c r="E52" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F52" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H52" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I52" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J52" s="2" t="s">
+      <c r="F52" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G52" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H52" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I52" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J52" s="5" t="s">
         <v>192</v>
       </c>
-      <c r="K52" s="2"/>
-      <c r="L52" s="2"/>
-      <c r="M52" s="2"/>
-    </row>
-    <row r="53" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K52" s="5"/>
+      <c r="L52" s="5"/>
+      <c r="M52" s="5"/>
+    </row>
+    <row r="53" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>137</v>
       </c>
@@ -4093,18 +3636,18 @@
       <c r="E53" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F53" s="2" t="s">
+      <c r="F53" s="5" t="s">
         <v>184</v>
       </c>
-      <c r="G53" s="2"/>
-      <c r="H53" s="2"/>
-      <c r="I53" s="2"/>
-      <c r="J53" s="2"/>
-      <c r="K53" s="2"/>
-      <c r="L53" s="2"/>
-      <c r="M53" s="2"/>
-    </row>
-    <row r="54" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G53" s="5"/>
+      <c r="H53" s="5"/>
+      <c r="I53" s="5"/>
+      <c r="J53" s="5"/>
+      <c r="K53" s="5"/>
+      <c r="L53" s="5"/>
+      <c r="M53" s="5"/>
+    </row>
+    <row r="54" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>138</v>
       </c>
@@ -4120,26 +3663,26 @@
       <c r="E54" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F54" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H54" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I54" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J54" s="2" t="s">
+      <c r="F54" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G54" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H54" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I54" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J54" s="5" t="s">
         <v>193</v>
       </c>
-      <c r="K54" s="2"/>
-      <c r="L54" s="2"/>
-      <c r="M54" s="2"/>
-    </row>
-    <row r="55" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K54" s="5"/>
+      <c r="L54" s="5"/>
+      <c r="M54" s="5"/>
+    </row>
+    <row r="55" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>139</v>
       </c>
@@ -4155,18 +3698,18 @@
       <c r="E55" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F55" s="2" t="s">
+      <c r="F55" s="5" t="s">
         <v>185</v>
       </c>
-      <c r="G55" s="2"/>
-      <c r="H55" s="2"/>
-      <c r="I55" s="2"/>
-      <c r="J55" s="2"/>
-      <c r="K55" s="2"/>
-      <c r="L55" s="2"/>
-      <c r="M55" s="2"/>
-    </row>
-    <row r="56" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G55" s="5"/>
+      <c r="H55" s="5"/>
+      <c r="I55" s="5"/>
+      <c r="J55" s="5"/>
+      <c r="K55" s="5"/>
+      <c r="L55" s="5"/>
+      <c r="M55" s="5"/>
+    </row>
+    <row r="56" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>140</v>
       </c>
@@ -4182,30 +3725,30 @@
       <c r="E56" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F56" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H56" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I56" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J56" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="K56" s="4" t="s">
-        <v>236</v>
+      <c r="F56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K56" s="3" t="s">
+        <v>235</v>
       </c>
       <c r="L56" s="6" t="s">
         <v>210</v>
       </c>
       <c r="M56" s="7"/>
     </row>
-    <row r="57" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>141</v>
       </c>
@@ -4221,18 +3764,18 @@
       <c r="E57" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F57" s="2" t="s">
+      <c r="F57" s="5" t="s">
         <v>189</v>
       </c>
-      <c r="G57" s="2"/>
-      <c r="H57" s="2"/>
-      <c r="I57" s="2"/>
-      <c r="J57" s="2"/>
-      <c r="K57" s="2"/>
-      <c r="L57" s="2"/>
-      <c r="M57" s="2"/>
-    </row>
-    <row r="58" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G57" s="5"/>
+      <c r="H57" s="5"/>
+      <c r="I57" s="5"/>
+      <c r="J57" s="5"/>
+      <c r="K57" s="5"/>
+      <c r="L57" s="5"/>
+      <c r="M57" s="5"/>
+    </row>
+    <row r="58" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>142</v>
       </c>
@@ -4248,26 +3791,26 @@
       <c r="E58" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F58" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H58" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I58" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J58" s="2" t="s">
+      <c r="F58" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G58" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H58" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I58" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J58" s="5" t="s">
         <v>195</v>
       </c>
-      <c r="K58" s="2"/>
-      <c r="L58" s="2"/>
-      <c r="M58" s="2"/>
-    </row>
-    <row r="59" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K58" s="5"/>
+      <c r="L58" s="5"/>
+      <c r="M58" s="5"/>
+    </row>
+    <row r="59" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>161</v>
       </c>
@@ -4283,18 +3826,18 @@
       <c r="E59" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="2" t="s">
+      <c r="F59" s="5" t="s">
         <v>187</v>
       </c>
-      <c r="G59" s="2"/>
-      <c r="H59" s="2"/>
-      <c r="I59" s="2"/>
-      <c r="J59" s="2"/>
-      <c r="K59" s="2"/>
-      <c r="L59" s="2"/>
-      <c r="M59" s="2"/>
-    </row>
-    <row r="60" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G59" s="5"/>
+      <c r="H59" s="5"/>
+      <c r="I59" s="5"/>
+      <c r="J59" s="5"/>
+      <c r="K59" s="5"/>
+      <c r="L59" s="5"/>
+      <c r="M59" s="5"/>
+    </row>
+    <row r="60" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>163</v>
       </c>
@@ -4310,26 +3853,26 @@
       <c r="E60" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F60" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H60" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I60" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J60" s="2" t="s">
+      <c r="F60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I60" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J60" s="5" t="s">
         <v>194</v>
       </c>
-      <c r="K60" s="2"/>
-      <c r="L60" s="2"/>
-      <c r="M60" s="2"/>
-    </row>
-    <row r="61" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K60" s="5"/>
+      <c r="L60" s="5"/>
+      <c r="M60" s="5"/>
+    </row>
+    <row r="61" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>165</v>
       </c>
@@ -4345,18 +3888,18 @@
       <c r="E61" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F61" s="2" t="s">
+      <c r="F61" s="5" t="s">
         <v>186</v>
       </c>
-      <c r="G61" s="2"/>
-      <c r="H61" s="2"/>
-      <c r="I61" s="2"/>
-      <c r="J61" s="2"/>
-      <c r="K61" s="2"/>
-      <c r="L61" s="2"/>
-      <c r="M61" s="2"/>
-    </row>
-    <row r="62" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="G61" s="5"/>
+      <c r="H61" s="5"/>
+      <c r="I61" s="5"/>
+      <c r="J61" s="5"/>
+      <c r="K61" s="5"/>
+      <c r="L61" s="5"/>
+      <c r="M61" s="5"/>
+    </row>
+    <row r="62" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>167</v>
       </c>
@@ -4372,26 +3915,26 @@
       <c r="E62" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F62" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="H62" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="I62" s="4" t="s">
-        <v>236</v>
-      </c>
-      <c r="J62" s="2" t="s">
+      <c r="F62" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G62" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H62" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I62" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J62" s="5" t="s">
         <v>196</v>
       </c>
-      <c r="K62" s="2"/>
-      <c r="L62" s="2"/>
-      <c r="M62" s="2"/>
-    </row>
-    <row r="63" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
+      <c r="K62" s="5"/>
+      <c r="L62" s="5"/>
+      <c r="M62" s="5"/>
+    </row>
+    <row r="63" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>169</v>
       </c>
@@ -4407,794 +3950,767 @@
       <c r="E63" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F63" s="2" t="s">
+      <c r="F63" s="5" t="s">
         <v>188</v>
       </c>
-      <c r="G63" s="2"/>
-      <c r="H63" s="2"/>
-      <c r="I63" s="2"/>
-      <c r="J63" s="2"/>
-      <c r="K63" s="2"/>
-      <c r="L63" s="2"/>
-      <c r="M63" s="2"/>
-    </row>
-    <row r="64" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="65" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="66" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="67" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="68" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="69" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="70" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="71" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="72" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="73" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4"/>
-    <row r="74" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E74" s="5"/>
-      <c r="F74" s="5"/>
-    </row>
-    <row r="75" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E75" s="5"/>
-      <c r="F75" s="5"/>
-    </row>
-    <row r="76" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E76" s="5"/>
-      <c r="F76" s="5"/>
-    </row>
-    <row r="77" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E77" s="5"/>
-      <c r="F77" s="5"/>
-    </row>
-    <row r="78" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E78" s="5"/>
-      <c r="F78" s="5"/>
-    </row>
-    <row r="79" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E79" s="5"/>
-      <c r="F79" s="5"/>
-    </row>
-    <row r="80" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E80" s="5"/>
-      <c r="F80" s="5"/>
-    </row>
-    <row r="81" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E81" s="5"/>
-      <c r="F81" s="5"/>
-    </row>
-    <row r="82" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E82" s="5"/>
-      <c r="F82" s="5"/>
-    </row>
-    <row r="83" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E83" s="5"/>
-      <c r="F83" s="5"/>
-    </row>
-    <row r="84" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E84" s="5"/>
-      <c r="F84" s="5"/>
-    </row>
-    <row r="85" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E85" s="5"/>
-      <c r="F85" s="5"/>
-    </row>
-    <row r="86" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E86" s="5"/>
-      <c r="F86" s="5"/>
-    </row>
-    <row r="87" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E87" s="5"/>
-      <c r="F87" s="5"/>
-    </row>
-    <row r="88" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E88" s="5"/>
-      <c r="F88" s="5"/>
-    </row>
-    <row r="89" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E89" s="5"/>
-      <c r="F89" s="5"/>
-    </row>
-    <row r="90" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E90" s="5"/>
-      <c r="F90" s="5"/>
-    </row>
-    <row r="91" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E91" s="5"/>
-      <c r="F91" s="5"/>
-    </row>
-    <row r="92" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E92" s="5"/>
-      <c r="F92" s="5"/>
-    </row>
-    <row r="93" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E93" s="5"/>
-      <c r="F93" s="5"/>
-    </row>
-    <row r="94" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E94" s="5"/>
-      <c r="F94" s="5"/>
-    </row>
-    <row r="95" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E95" s="5"/>
-      <c r="F95" s="5"/>
-    </row>
-    <row r="96" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E96" s="5"/>
-      <c r="F96" s="5"/>
-    </row>
-    <row r="97" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E97" s="5"/>
-      <c r="F97" s="5"/>
-    </row>
-    <row r="98" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E98" s="5"/>
-      <c r="F98" s="5"/>
-    </row>
-    <row r="99" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E99" s="5"/>
-      <c r="F99" s="5"/>
-    </row>
-    <row r="100" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E100" s="5"/>
-      <c r="F100" s="5"/>
-    </row>
-    <row r="101" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E101" s="5"/>
-      <c r="F101" s="5"/>
-    </row>
-    <row r="102" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E102" s="5"/>
-      <c r="F102" s="5"/>
-    </row>
-    <row r="103" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E103" s="5"/>
-      <c r="F103" s="5"/>
-    </row>
-    <row r="104" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E104" s="5"/>
-      <c r="F104" s="5"/>
-    </row>
-    <row r="105" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E105" s="5"/>
-      <c r="F105" s="5"/>
-    </row>
-    <row r="106" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E106" s="5"/>
-      <c r="F106" s="5"/>
-    </row>
-    <row r="107" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E107" s="5"/>
-      <c r="F107" s="5"/>
-    </row>
-    <row r="108" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E108" s="5"/>
-      <c r="F108" s="5"/>
-    </row>
-    <row r="109" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E109" s="5"/>
-      <c r="F109" s="5"/>
-    </row>
-    <row r="110" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E110" s="5"/>
-      <c r="F110" s="5"/>
-    </row>
-    <row r="111" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E111" s="5"/>
-      <c r="F111" s="5"/>
-    </row>
-    <row r="112" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E112" s="5"/>
-      <c r="F112" s="5"/>
-    </row>
-    <row r="113" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E113" s="5"/>
-      <c r="F113" s="5"/>
-    </row>
-    <row r="114" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E114" s="5"/>
-      <c r="F114" s="5"/>
-    </row>
-    <row r="115" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E115" s="5"/>
-      <c r="F115" s="5"/>
-    </row>
-    <row r="116" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E116" s="5"/>
-      <c r="F116" s="5"/>
-    </row>
-    <row r="117" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E117" s="5"/>
-      <c r="F117" s="5"/>
-    </row>
-    <row r="118" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E118" s="5"/>
-      <c r="F118" s="5"/>
-    </row>
-    <row r="119" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E119" s="5"/>
-      <c r="F119" s="5"/>
-    </row>
-    <row r="120" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E120" s="5"/>
-      <c r="F120" s="5"/>
-    </row>
-    <row r="121" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E121" s="5"/>
-      <c r="F121" s="5"/>
-      <c r="G121" s="5"/>
-    </row>
-    <row r="122" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E122" s="5"/>
-      <c r="F122" s="5"/>
-      <c r="G122" s="5"/>
-    </row>
-    <row r="123" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E123" s="5"/>
-      <c r="F123" s="5"/>
-      <c r="G123" s="5"/>
-    </row>
-    <row r="124" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E124" s="5"/>
-      <c r="F124" s="5"/>
-      <c r="G124" s="5"/>
-    </row>
-    <row r="125" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E125" s="5"/>
-      <c r="F125" s="5"/>
-      <c r="G125" s="5"/>
-    </row>
-    <row r="126" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E126" s="5"/>
-      <c r="F126" s="5"/>
-    </row>
-    <row r="127" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E127" s="5"/>
-      <c r="F127" s="5"/>
-    </row>
-    <row r="128" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E128" s="5"/>
-      <c r="F128" s="5"/>
-      <c r="G128" s="5"/>
-    </row>
-    <row r="129" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E129" s="5"/>
-      <c r="F129" s="5"/>
-      <c r="G129" s="5"/>
-    </row>
-    <row r="130" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E130" s="5"/>
-      <c r="F130" s="5"/>
-    </row>
-    <row r="131" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E131" s="5"/>
-      <c r="F131" s="5"/>
-      <c r="G131" s="5"/>
-    </row>
-    <row r="132" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E132" s="5"/>
-      <c r="F132" s="5"/>
-    </row>
-    <row r="133" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E133" s="5"/>
-      <c r="F133" s="5"/>
-      <c r="G133" s="5"/>
-    </row>
-    <row r="134" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E134" s="5"/>
-      <c r="F134" s="5"/>
-    </row>
-    <row r="135" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E135" s="5"/>
-      <c r="F135" s="5"/>
-    </row>
-    <row r="136" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E136" s="5"/>
-      <c r="F136" s="5"/>
-    </row>
-    <row r="137" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E137" s="5"/>
-      <c r="F137" s="5"/>
-    </row>
-    <row r="138" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E138" s="5"/>
-      <c r="F138" s="5"/>
-    </row>
-    <row r="139" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E139" s="5"/>
-      <c r="F139" s="5"/>
-    </row>
-    <row r="140" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E140" s="5"/>
-      <c r="F140" s="5"/>
-      <c r="G140" s="5"/>
-    </row>
-    <row r="141" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E141" s="5"/>
-      <c r="F141" s="5"/>
-      <c r="G141" s="5"/>
-    </row>
-    <row r="142" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E142" s="5"/>
-      <c r="F142" s="5"/>
-    </row>
-    <row r="143" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E143" s="5"/>
-      <c r="F143" s="5"/>
-      <c r="G143" s="5"/>
-    </row>
-    <row r="144" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E144" s="5"/>
-      <c r="F144" s="5"/>
-      <c r="G144" s="5"/>
-    </row>
-    <row r="145" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E145" s="5"/>
-      <c r="F145" s="5"/>
-      <c r="G145" s="5"/>
-    </row>
-    <row r="146" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E146" s="5"/>
-      <c r="F146" s="5"/>
-      <c r="G146" s="5"/>
-    </row>
-    <row r="147" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E147" s="5"/>
-      <c r="F147" s="5"/>
-    </row>
-    <row r="148" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E148" s="5"/>
-      <c r="F148" s="5"/>
-    </row>
-    <row r="149" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E149" s="5"/>
-      <c r="F149" s="5"/>
-    </row>
-    <row r="150" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E150" s="5"/>
-      <c r="F150" s="5"/>
-    </row>
-    <row r="151" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E151" s="5"/>
-      <c r="F151" s="5"/>
-    </row>
-    <row r="152" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E152" s="5"/>
-      <c r="F152" s="5"/>
-    </row>
-    <row r="153" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E153" s="5"/>
-      <c r="F153" s="5"/>
-    </row>
-    <row r="154" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E154" s="5"/>
-      <c r="F154" s="5"/>
-    </row>
-    <row r="155" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E155" s="5"/>
-      <c r="F155" s="5"/>
-    </row>
-    <row r="156" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E156" s="5"/>
-      <c r="F156" s="5"/>
-      <c r="G156" s="5"/>
-    </row>
-    <row r="157" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E157" s="5"/>
-      <c r="F157" s="5"/>
-      <c r="G157" s="5"/>
-    </row>
-    <row r="158" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E158" s="5"/>
-      <c r="F158" s="5"/>
-      <c r="G158" s="5"/>
-    </row>
-    <row r="159" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E159" s="5"/>
-      <c r="F159" s="5"/>
-      <c r="G159" s="5"/>
-    </row>
-    <row r="160" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E160" s="5"/>
-      <c r="F160" s="5"/>
-    </row>
-    <row r="161" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E161" s="5"/>
-      <c r="F161" s="5"/>
-    </row>
-    <row r="162" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E162" s="5"/>
-      <c r="F162" s="5"/>
-    </row>
-    <row r="163" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E163" s="5"/>
-      <c r="F163" s="5"/>
-    </row>
-    <row r="164" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E164" s="5"/>
-      <c r="F164" s="5"/>
-    </row>
-    <row r="165" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E165" s="5"/>
-      <c r="F165" s="5"/>
-    </row>
-    <row r="166" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E166" s="5"/>
-      <c r="F166" s="5"/>
-    </row>
-    <row r="167" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E167" s="5"/>
-      <c r="F167" s="5"/>
-    </row>
-    <row r="168" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E168" s="5"/>
-      <c r="F168" s="5"/>
-    </row>
-    <row r="169" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E169" s="5"/>
-      <c r="F169" s="5"/>
-    </row>
-    <row r="170" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E170" s="5"/>
-      <c r="F170" s="5"/>
-    </row>
-    <row r="171" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E171" s="5"/>
-      <c r="F171" s="5"/>
-    </row>
-    <row r="172" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E172" s="5"/>
-      <c r="F172" s="5"/>
-    </row>
-    <row r="173" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E173" s="5"/>
-      <c r="F173" s="5"/>
-    </row>
-    <row r="174" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E174" s="5"/>
-      <c r="F174" s="5"/>
-    </row>
-    <row r="175" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E175" s="5"/>
-      <c r="F175" s="5"/>
-    </row>
-    <row r="176" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E176" s="5"/>
-      <c r="F176" s="5"/>
-    </row>
-    <row r="177" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E177" s="5"/>
-      <c r="F177" s="5"/>
-    </row>
-    <row r="178" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E178" s="5"/>
-      <c r="F178" s="5"/>
-    </row>
-    <row r="179" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E179" s="5"/>
-      <c r="F179" s="5"/>
-    </row>
-    <row r="180" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E180" s="5"/>
-      <c r="F180" s="5"/>
-    </row>
-    <row r="181" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E181" s="5"/>
-      <c r="F181" s="5"/>
-    </row>
-    <row r="182" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E182" s="5"/>
-      <c r="F182" s="5"/>
-    </row>
-    <row r="183" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E183" s="5"/>
-      <c r="F183" s="5"/>
-    </row>
-    <row r="184" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E184" s="5"/>
-      <c r="F184" s="5"/>
-    </row>
-    <row r="185" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E185" s="5"/>
-      <c r="F185" s="5"/>
-    </row>
-    <row r="186" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E186" s="5"/>
-      <c r="F186" s="5"/>
-    </row>
-    <row r="187" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E187" s="5"/>
-      <c r="F187" s="5"/>
-      <c r="G187" s="5"/>
-    </row>
-    <row r="188" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E188" s="5"/>
-      <c r="F188" s="5"/>
-    </row>
-    <row r="189" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E189" s="5"/>
-      <c r="F189" s="5"/>
-    </row>
-    <row r="190" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E190" s="5"/>
-      <c r="F190" s="5"/>
-      <c r="G190" s="5"/>
-    </row>
-    <row r="191" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E191" s="5"/>
-      <c r="F191" s="5"/>
-    </row>
-    <row r="192" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E192" s="5"/>
-      <c r="F192" s="5"/>
-      <c r="G192" s="5"/>
-    </row>
-    <row r="193" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E193" s="5"/>
-      <c r="F193" s="5"/>
-      <c r="G193" s="5"/>
-    </row>
-    <row r="194" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E194" s="5"/>
-      <c r="F194" s="5"/>
-      <c r="G194" s="5"/>
-    </row>
-    <row r="195" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E195" s="5"/>
-      <c r="F195" s="5"/>
-    </row>
-    <row r="196" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E196" s="5"/>
-      <c r="F196" s="5"/>
-      <c r="G196" s="5"/>
-    </row>
-    <row r="197" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E197" s="5"/>
-      <c r="F197" s="5"/>
-    </row>
-    <row r="198" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E198" s="5"/>
-      <c r="F198" s="5"/>
-      <c r="G198" s="5"/>
-    </row>
-    <row r="199" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E199" s="5"/>
-      <c r="F199" s="5"/>
-      <c r="G199" s="5"/>
-    </row>
-    <row r="200" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E200" s="5"/>
-      <c r="F200" s="5"/>
-      <c r="G200" s="5"/>
-    </row>
-    <row r="201" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E201" s="5"/>
-      <c r="F201" s="5"/>
-      <c r="G201" s="5"/>
-    </row>
-    <row r="202" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E202" s="5"/>
-      <c r="F202" s="5"/>
-    </row>
-    <row r="203" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E203" s="5"/>
-      <c r="F203" s="5"/>
-    </row>
-    <row r="204" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E204" s="5"/>
-      <c r="F204" s="5"/>
-    </row>
-    <row r="205" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E205" s="5"/>
-      <c r="F205" s="5"/>
-    </row>
-    <row r="206" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E206" s="5"/>
-      <c r="F206" s="5"/>
-    </row>
-    <row r="207" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E207" s="5"/>
-      <c r="F207" s="5"/>
-    </row>
-    <row r="208" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E208" s="5"/>
-      <c r="F208" s="5"/>
-    </row>
-    <row r="209" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E209" s="5"/>
-      <c r="F209" s="5"/>
-    </row>
-    <row r="210" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E210" s="5"/>
-      <c r="F210" s="5"/>
-    </row>
-    <row r="211" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E211" s="5"/>
-      <c r="F211" s="5"/>
-    </row>
-    <row r="212" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E212" s="5"/>
-      <c r="F212" s="5"/>
-      <c r="G212" s="5"/>
-    </row>
-    <row r="213" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E213" s="5"/>
-      <c r="F213" s="5"/>
-    </row>
-    <row r="214" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E214" s="5"/>
-      <c r="F214" s="5"/>
-    </row>
-    <row r="215" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E215" s="5"/>
-      <c r="F215" s="5"/>
-    </row>
-    <row r="216" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E216" s="5"/>
-      <c r="F216" s="5"/>
-    </row>
-    <row r="217" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E217" s="5"/>
-      <c r="F217" s="5"/>
-      <c r="G217" s="5"/>
-    </row>
-    <row r="218" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E218" s="5"/>
-      <c r="F218" s="5"/>
-    </row>
-    <row r="219" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E219" s="5"/>
-      <c r="F219" s="5"/>
-    </row>
-    <row r="220" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E220" s="5"/>
-      <c r="F220" s="5"/>
-    </row>
-    <row r="221" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E221" s="5"/>
-      <c r="F221" s="5"/>
-    </row>
-    <row r="222" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E222" s="5"/>
-      <c r="F222" s="5"/>
-      <c r="G222" s="5"/>
-    </row>
-    <row r="223" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E223" s="5"/>
-      <c r="F223" s="5"/>
-      <c r="G223" s="5"/>
-    </row>
-    <row r="224" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E224" s="5"/>
-      <c r="F224" s="5"/>
-    </row>
-    <row r="225" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E225" s="5"/>
-      <c r="F225" s="5"/>
-    </row>
-    <row r="226" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E226" s="5"/>
-      <c r="F226" s="5"/>
-    </row>
-    <row r="227" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E227" s="5"/>
-      <c r="F227" s="5"/>
-    </row>
-    <row r="228" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E228" s="5"/>
-      <c r="F228" s="5"/>
-    </row>
-    <row r="229" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E229" s="5"/>
-      <c r="F229" s="5"/>
-    </row>
-    <row r="230" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E230" s="5"/>
-      <c r="F230" s="5"/>
-    </row>
-    <row r="231" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E231" s="5"/>
-      <c r="F231" s="5"/>
-    </row>
-    <row r="232" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E232" s="5"/>
-      <c r="F232" s="5"/>
-    </row>
-    <row r="233" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E233" s="5"/>
-      <c r="F233" s="5"/>
-    </row>
-    <row r="234" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E234" s="5"/>
-      <c r="F234" s="5"/>
-    </row>
-    <row r="235" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E235" s="5"/>
-      <c r="F235" s="5"/>
-    </row>
-    <row r="236" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E236" s="5"/>
-      <c r="F236" s="5"/>
-    </row>
-    <row r="237" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E237" s="5"/>
-      <c r="F237" s="5"/>
-    </row>
-    <row r="238" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E238" s="5"/>
-      <c r="F238" s="5"/>
-      <c r="G238" s="5"/>
-    </row>
-    <row r="239" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E239" s="5"/>
-      <c r="F239" s="5"/>
-      <c r="G239" s="5"/>
-    </row>
-    <row r="240" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E240" s="5"/>
-      <c r="F240" s="5"/>
-    </row>
-    <row r="241" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E241" s="5"/>
-      <c r="F241" s="5"/>
-    </row>
-    <row r="242" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E242" s="5"/>
-      <c r="F242" s="5"/>
-      <c r="G242" s="5"/>
-    </row>
-    <row r="243" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E243" s="5"/>
-      <c r="F243" s="5"/>
-      <c r="G243" s="5"/>
-    </row>
-    <row r="244" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E244" s="5"/>
-      <c r="F244" s="5"/>
-    </row>
-    <row r="245" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E245" s="5"/>
-      <c r="F245" s="5"/>
-      <c r="G245" s="5"/>
-    </row>
-    <row r="246" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="E246" s="5"/>
-      <c r="F246" s="5"/>
-      <c r="G246" s="5"/>
+      <c r="G63" s="5"/>
+      <c r="H63" s="5"/>
+      <c r="I63" s="5"/>
+      <c r="J63" s="5"/>
+      <c r="K63" s="5"/>
+      <c r="L63" s="5"/>
+      <c r="M63" s="5"/>
+    </row>
+    <row r="64" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="65" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="66" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="67" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="68" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="69" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="70" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="71" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="72" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="73" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="74" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E74" s="4"/>
+      <c r="F74" s="4"/>
+    </row>
+    <row r="75" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E75" s="4"/>
+      <c r="F75" s="4"/>
+    </row>
+    <row r="76" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E76" s="4"/>
+      <c r="F76" s="4"/>
+    </row>
+    <row r="77" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E77" s="4"/>
+      <c r="F77" s="4"/>
+    </row>
+    <row r="78" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E78" s="4"/>
+      <c r="F78" s="4"/>
+    </row>
+    <row r="79" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E79" s="4"/>
+      <c r="F79" s="4"/>
+    </row>
+    <row r="80" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E80" s="4"/>
+      <c r="F80" s="4"/>
+    </row>
+    <row r="81" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E81" s="4"/>
+      <c r="F81" s="4"/>
+    </row>
+    <row r="82" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E82" s="4"/>
+      <c r="F82" s="4"/>
+    </row>
+    <row r="83" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E83" s="4"/>
+      <c r="F83" s="4"/>
+    </row>
+    <row r="84" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E84" s="4"/>
+      <c r="F84" s="4"/>
+    </row>
+    <row r="85" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E85" s="4"/>
+      <c r="F85" s="4"/>
+    </row>
+    <row r="86" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E86" s="4"/>
+      <c r="F86" s="4"/>
+    </row>
+    <row r="87" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E87" s="4"/>
+      <c r="F87" s="4"/>
+    </row>
+    <row r="88" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E88" s="4"/>
+      <c r="F88" s="4"/>
+    </row>
+    <row r="89" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E89" s="4"/>
+      <c r="F89" s="4"/>
+    </row>
+    <row r="90" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E90" s="4"/>
+      <c r="F90" s="4"/>
+    </row>
+    <row r="91" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E91" s="4"/>
+      <c r="F91" s="4"/>
+    </row>
+    <row r="92" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E92" s="4"/>
+      <c r="F92" s="4"/>
+    </row>
+    <row r="93" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E93" s="4"/>
+      <c r="F93" s="4"/>
+    </row>
+    <row r="94" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E94" s="4"/>
+      <c r="F94" s="4"/>
+    </row>
+    <row r="95" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E95" s="4"/>
+      <c r="F95" s="4"/>
+    </row>
+    <row r="96" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E96" s="4"/>
+      <c r="F96" s="4"/>
+    </row>
+    <row r="97" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E97" s="4"/>
+      <c r="F97" s="4"/>
+    </row>
+    <row r="98" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+    </row>
+    <row r="99" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+    </row>
+    <row r="100" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
+    </row>
+    <row r="101" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E101" s="4"/>
+      <c r="F101" s="4"/>
+    </row>
+    <row r="102" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E102" s="4"/>
+      <c r="F102" s="4"/>
+    </row>
+    <row r="103" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E103" s="4"/>
+      <c r="F103" s="4"/>
+    </row>
+    <row r="104" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E104" s="4"/>
+      <c r="F104" s="4"/>
+    </row>
+    <row r="105" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E105" s="4"/>
+      <c r="F105" s="4"/>
+    </row>
+    <row r="106" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E106" s="4"/>
+      <c r="F106" s="4"/>
+    </row>
+    <row r="107" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E107" s="4"/>
+      <c r="F107" s="4"/>
+    </row>
+    <row r="108" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E108" s="4"/>
+      <c r="F108" s="4"/>
+    </row>
+    <row r="109" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E109" s="4"/>
+      <c r="F109" s="4"/>
+    </row>
+    <row r="110" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E110" s="4"/>
+      <c r="F110" s="4"/>
+    </row>
+    <row r="111" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E111" s="4"/>
+      <c r="F111" s="4"/>
+    </row>
+    <row r="112" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E112" s="4"/>
+      <c r="F112" s="4"/>
+    </row>
+    <row r="113" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E113" s="4"/>
+      <c r="F113" s="4"/>
+    </row>
+    <row r="114" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E114" s="4"/>
+      <c r="F114" s="4"/>
+    </row>
+    <row r="115" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E115" s="4"/>
+      <c r="F115" s="4"/>
+    </row>
+    <row r="116" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E116" s="4"/>
+      <c r="F116" s="4"/>
+    </row>
+    <row r="117" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E117" s="4"/>
+      <c r="F117" s="4"/>
+    </row>
+    <row r="118" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E118" s="4"/>
+      <c r="F118" s="4"/>
+    </row>
+    <row r="119" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E119" s="4"/>
+      <c r="F119" s="4"/>
+    </row>
+    <row r="120" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E120" s="4"/>
+      <c r="F120" s="4"/>
+    </row>
+    <row r="121" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E121" s="4"/>
+      <c r="F121" s="4"/>
+      <c r="G121" s="4"/>
+    </row>
+    <row r="122" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E122" s="4"/>
+      <c r="F122" s="4"/>
+      <c r="G122" s="4"/>
+    </row>
+    <row r="123" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E123" s="4"/>
+      <c r="F123" s="4"/>
+      <c r="G123" s="4"/>
+    </row>
+    <row r="124" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E124" s="4"/>
+      <c r="F124" s="4"/>
+      <c r="G124" s="4"/>
+    </row>
+    <row r="125" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E125" s="4"/>
+      <c r="F125" s="4"/>
+      <c r="G125" s="4"/>
+    </row>
+    <row r="126" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E126" s="4"/>
+      <c r="F126" s="4"/>
+    </row>
+    <row r="127" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E127" s="4"/>
+      <c r="F127" s="4"/>
+    </row>
+    <row r="128" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E128" s="4"/>
+      <c r="F128" s="4"/>
+      <c r="G128" s="4"/>
+    </row>
+    <row r="129" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E129" s="4"/>
+      <c r="F129" s="4"/>
+      <c r="G129" s="4"/>
+    </row>
+    <row r="130" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E130" s="4"/>
+      <c r="F130" s="4"/>
+    </row>
+    <row r="131" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E131" s="4"/>
+      <c r="F131" s="4"/>
+      <c r="G131" s="4"/>
+    </row>
+    <row r="132" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E132" s="4"/>
+      <c r="F132" s="4"/>
+    </row>
+    <row r="133" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E133" s="4"/>
+      <c r="F133" s="4"/>
+      <c r="G133" s="4"/>
+    </row>
+    <row r="134" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E134" s="4"/>
+      <c r="F134" s="4"/>
+    </row>
+    <row r="135" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E135" s="4"/>
+      <c r="F135" s="4"/>
+    </row>
+    <row r="136" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E136" s="4"/>
+      <c r="F136" s="4"/>
+    </row>
+    <row r="137" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E137" s="4"/>
+      <c r="F137" s="4"/>
+    </row>
+    <row r="138" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E138" s="4"/>
+      <c r="F138" s="4"/>
+    </row>
+    <row r="139" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E139" s="4"/>
+      <c r="F139" s="4"/>
+    </row>
+    <row r="140" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E140" s="4"/>
+      <c r="F140" s="4"/>
+      <c r="G140" s="4"/>
+    </row>
+    <row r="141" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E141" s="4"/>
+      <c r="F141" s="4"/>
+      <c r="G141" s="4"/>
+    </row>
+    <row r="142" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E142" s="4"/>
+      <c r="F142" s="4"/>
+    </row>
+    <row r="143" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E143" s="4"/>
+      <c r="F143" s="4"/>
+      <c r="G143" s="4"/>
+    </row>
+    <row r="144" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E144" s="4"/>
+      <c r="F144" s="4"/>
+      <c r="G144" s="4"/>
+    </row>
+    <row r="145" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E145" s="4"/>
+      <c r="F145" s="4"/>
+      <c r="G145" s="4"/>
+    </row>
+    <row r="146" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E146" s="4"/>
+      <c r="F146" s="4"/>
+      <c r="G146" s="4"/>
+    </row>
+    <row r="147" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E147" s="4"/>
+      <c r="F147" s="4"/>
+    </row>
+    <row r="148" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E148" s="4"/>
+      <c r="F148" s="4"/>
+    </row>
+    <row r="149" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E149" s="4"/>
+      <c r="F149" s="4"/>
+    </row>
+    <row r="150" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E150" s="4"/>
+      <c r="F150" s="4"/>
+    </row>
+    <row r="151" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E151" s="4"/>
+      <c r="F151" s="4"/>
+    </row>
+    <row r="152" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E152" s="4"/>
+      <c r="F152" s="4"/>
+    </row>
+    <row r="153" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E153" s="4"/>
+      <c r="F153" s="4"/>
+    </row>
+    <row r="154" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E154" s="4"/>
+      <c r="F154" s="4"/>
+    </row>
+    <row r="155" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E155" s="4"/>
+      <c r="F155" s="4"/>
+    </row>
+    <row r="156" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E156" s="4"/>
+      <c r="F156" s="4"/>
+      <c r="G156" s="4"/>
+    </row>
+    <row r="157" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E157" s="4"/>
+      <c r="F157" s="4"/>
+      <c r="G157" s="4"/>
+    </row>
+    <row r="158" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E158" s="4"/>
+      <c r="F158" s="4"/>
+      <c r="G158" s="4"/>
+    </row>
+    <row r="159" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E159" s="4"/>
+      <c r="F159" s="4"/>
+      <c r="G159" s="4"/>
+    </row>
+    <row r="160" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E160" s="4"/>
+      <c r="F160" s="4"/>
+    </row>
+    <row r="161" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E161" s="4"/>
+      <c r="F161" s="4"/>
+    </row>
+    <row r="162" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E162" s="4"/>
+      <c r="F162" s="4"/>
+    </row>
+    <row r="163" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E163" s="4"/>
+      <c r="F163" s="4"/>
+    </row>
+    <row r="164" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E164" s="4"/>
+      <c r="F164" s="4"/>
+    </row>
+    <row r="165" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E165" s="4"/>
+      <c r="F165" s="4"/>
+    </row>
+    <row r="166" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E166" s="4"/>
+      <c r="F166" s="4"/>
+    </row>
+    <row r="167" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E167" s="4"/>
+      <c r="F167" s="4"/>
+    </row>
+    <row r="168" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E168" s="4"/>
+      <c r="F168" s="4"/>
+    </row>
+    <row r="169" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E169" s="4"/>
+      <c r="F169" s="4"/>
+    </row>
+    <row r="170" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E170" s="4"/>
+      <c r="F170" s="4"/>
+    </row>
+    <row r="171" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E171" s="4"/>
+      <c r="F171" s="4"/>
+    </row>
+    <row r="172" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E172" s="4"/>
+      <c r="F172" s="4"/>
+    </row>
+    <row r="173" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E173" s="4"/>
+      <c r="F173" s="4"/>
+    </row>
+    <row r="174" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E174" s="4"/>
+      <c r="F174" s="4"/>
+    </row>
+    <row r="175" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E175" s="4"/>
+      <c r="F175" s="4"/>
+    </row>
+    <row r="176" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E176" s="4"/>
+      <c r="F176" s="4"/>
+    </row>
+    <row r="177" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E177" s="4"/>
+      <c r="F177" s="4"/>
+    </row>
+    <row r="178" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E178" s="4"/>
+      <c r="F178" s="4"/>
+    </row>
+    <row r="179" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E179" s="4"/>
+      <c r="F179" s="4"/>
+    </row>
+    <row r="180" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E180" s="4"/>
+      <c r="F180" s="4"/>
+    </row>
+    <row r="181" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E181" s="4"/>
+      <c r="F181" s="4"/>
+    </row>
+    <row r="182" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E182" s="4"/>
+      <c r="F182" s="4"/>
+    </row>
+    <row r="183" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E183" s="4"/>
+      <c r="F183" s="4"/>
+    </row>
+    <row r="184" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E184" s="4"/>
+      <c r="F184" s="4"/>
+    </row>
+    <row r="185" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E185" s="4"/>
+      <c r="F185" s="4"/>
+    </row>
+    <row r="186" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E186" s="4"/>
+      <c r="F186" s="4"/>
+    </row>
+    <row r="187" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E187" s="4"/>
+      <c r="F187" s="4"/>
+      <c r="G187" s="4"/>
+    </row>
+    <row r="188" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E188" s="4"/>
+      <c r="F188" s="4"/>
+    </row>
+    <row r="189" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E189" s="4"/>
+      <c r="F189" s="4"/>
+    </row>
+    <row r="190" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E190" s="4"/>
+      <c r="F190" s="4"/>
+      <c r="G190" s="4"/>
+    </row>
+    <row r="191" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E191" s="4"/>
+      <c r="F191" s="4"/>
+    </row>
+    <row r="192" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E192" s="4"/>
+      <c r="F192" s="4"/>
+      <c r="G192" s="4"/>
+    </row>
+    <row r="193" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E193" s="4"/>
+      <c r="F193" s="4"/>
+      <c r="G193" s="4"/>
+    </row>
+    <row r="194" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E194" s="4"/>
+      <c r="F194" s="4"/>
+      <c r="G194" s="4"/>
+    </row>
+    <row r="195" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E195" s="4"/>
+      <c r="F195" s="4"/>
+    </row>
+    <row r="196" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E196" s="4"/>
+      <c r="F196" s="4"/>
+      <c r="G196" s="4"/>
+    </row>
+    <row r="197" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E197" s="4"/>
+      <c r="F197" s="4"/>
+    </row>
+    <row r="198" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E198" s="4"/>
+      <c r="F198" s="4"/>
+      <c r="G198" s="4"/>
+    </row>
+    <row r="199" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E199" s="4"/>
+      <c r="F199" s="4"/>
+      <c r="G199" s="4"/>
+    </row>
+    <row r="200" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E200" s="4"/>
+      <c r="F200" s="4"/>
+      <c r="G200" s="4"/>
+    </row>
+    <row r="201" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E201" s="4"/>
+      <c r="F201" s="4"/>
+      <c r="G201" s="4"/>
+    </row>
+    <row r="202" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E202" s="4"/>
+      <c r="F202" s="4"/>
+    </row>
+    <row r="203" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E203" s="4"/>
+      <c r="F203" s="4"/>
+    </row>
+    <row r="204" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E204" s="4"/>
+      <c r="F204" s="4"/>
+    </row>
+    <row r="205" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E205" s="4"/>
+      <c r="F205" s="4"/>
+    </row>
+    <row r="206" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E206" s="4"/>
+      <c r="F206" s="4"/>
+    </row>
+    <row r="207" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E207" s="4"/>
+      <c r="F207" s="4"/>
+    </row>
+    <row r="208" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E208" s="4"/>
+      <c r="F208" s="4"/>
+    </row>
+    <row r="209" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E209" s="4"/>
+      <c r="F209" s="4"/>
+    </row>
+    <row r="210" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E210" s="4"/>
+      <c r="F210" s="4"/>
+    </row>
+    <row r="211" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E211" s="4"/>
+      <c r="F211" s="4"/>
+    </row>
+    <row r="212" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E212" s="4"/>
+      <c r="F212" s="4"/>
+      <c r="G212" s="4"/>
+    </row>
+    <row r="213" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E213" s="4"/>
+      <c r="F213" s="4"/>
+    </row>
+    <row r="214" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E214" s="4"/>
+      <c r="F214" s="4"/>
+    </row>
+    <row r="215" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E215" s="4"/>
+      <c r="F215" s="4"/>
+    </row>
+    <row r="216" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E216" s="4"/>
+      <c r="F216" s="4"/>
+    </row>
+    <row r="217" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E217" s="4"/>
+      <c r="F217" s="4"/>
+      <c r="G217" s="4"/>
+    </row>
+    <row r="218" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E218" s="4"/>
+      <c r="F218" s="4"/>
+    </row>
+    <row r="219" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E219" s="4"/>
+      <c r="F219" s="4"/>
+    </row>
+    <row r="220" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E220" s="4"/>
+      <c r="F220" s="4"/>
+    </row>
+    <row r="221" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E221" s="4"/>
+      <c r="F221" s="4"/>
+    </row>
+    <row r="222" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E222" s="4"/>
+      <c r="F222" s="4"/>
+      <c r="G222" s="4"/>
+    </row>
+    <row r="223" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E223" s="4"/>
+      <c r="F223" s="4"/>
+      <c r="G223" s="4"/>
+    </row>
+    <row r="224" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E224" s="4"/>
+      <c r="F224" s="4"/>
+    </row>
+    <row r="225" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E225" s="4"/>
+      <c r="F225" s="4"/>
+    </row>
+    <row r="226" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E226" s="4"/>
+      <c r="F226" s="4"/>
+    </row>
+    <row r="227" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E227" s="4"/>
+      <c r="F227" s="4"/>
+    </row>
+    <row r="228" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E228" s="4"/>
+      <c r="F228" s="4"/>
+    </row>
+    <row r="229" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E229" s="4"/>
+      <c r="F229" s="4"/>
+    </row>
+    <row r="230" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E230" s="4"/>
+      <c r="F230" s="4"/>
+    </row>
+    <row r="231" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E231" s="4"/>
+      <c r="F231" s="4"/>
+    </row>
+    <row r="232" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E232" s="4"/>
+      <c r="F232" s="4"/>
+    </row>
+    <row r="233" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E233" s="4"/>
+      <c r="F233" s="4"/>
+    </row>
+    <row r="234" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E234" s="4"/>
+      <c r="F234" s="4"/>
+    </row>
+    <row r="235" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E235" s="4"/>
+      <c r="F235" s="4"/>
+    </row>
+    <row r="236" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E236" s="4"/>
+      <c r="F236" s="4"/>
+    </row>
+    <row r="237" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E237" s="4"/>
+      <c r="F237" s="4"/>
+    </row>
+    <row r="238" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E238" s="4"/>
+      <c r="F238" s="4"/>
+      <c r="G238" s="4"/>
+    </row>
+    <row r="239" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E239" s="4"/>
+      <c r="F239" s="4"/>
+      <c r="G239" s="4"/>
+    </row>
+    <row r="240" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E240" s="4"/>
+      <c r="F240" s="4"/>
+    </row>
+    <row r="241" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E241" s="4"/>
+      <c r="F241" s="4"/>
+    </row>
+    <row r="242" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E242" s="4"/>
+      <c r="F242" s="4"/>
+      <c r="G242" s="4"/>
+    </row>
+    <row r="243" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E243" s="4"/>
+      <c r="F243" s="4"/>
+      <c r="G243" s="4"/>
+    </row>
+    <row r="244" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E244" s="4"/>
+      <c r="F244" s="4"/>
+    </row>
+    <row r="245" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E245" s="4"/>
+      <c r="F245" s="4"/>
+      <c r="G245" s="4"/>
+    </row>
+    <row r="246" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E246" s="4"/>
+      <c r="F246" s="4"/>
+      <c r="G246" s="4"/>
     </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="J44:M44"/>
-    <mergeCell ref="F45:M45"/>
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="J40:K40"/>
-    <mergeCell ref="F41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="F35:M35"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="K36:M36"/>
-    <mergeCell ref="I37:J37"/>
-    <mergeCell ref="K37:M37"/>
-    <mergeCell ref="F1:M1"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J22:M22"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="F28:M28"/>
-    <mergeCell ref="F29:M29"/>
-    <mergeCell ref="G30:M30"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="F32:M32"/>
-    <mergeCell ref="G33:M33"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="J62:M62"/>
+    <mergeCell ref="F63:M63"/>
+    <mergeCell ref="F57:M57"/>
+    <mergeCell ref="J58:M58"/>
+    <mergeCell ref="F59:M59"/>
+    <mergeCell ref="J60:M60"/>
+    <mergeCell ref="F61:M61"/>
     <mergeCell ref="H38:M38"/>
     <mergeCell ref="F51:M51"/>
     <mergeCell ref="J52:M52"/>
@@ -5206,15 +4722,42 @@
     <mergeCell ref="J50:M50"/>
     <mergeCell ref="F40:G40"/>
     <mergeCell ref="H40:I40"/>
+    <mergeCell ref="G33:M33"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="G34:I34"/>
+    <mergeCell ref="L34:M34"/>
+    <mergeCell ref="F28:M28"/>
+    <mergeCell ref="F29:M29"/>
+    <mergeCell ref="G30:M30"/>
+    <mergeCell ref="L31:M31"/>
+    <mergeCell ref="F32:M32"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="J22:M22"/>
+    <mergeCell ref="L24:M24"/>
+    <mergeCell ref="L27:M27"/>
+    <mergeCell ref="F1:M1"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="F35:M35"/>
+    <mergeCell ref="G36:H36"/>
+    <mergeCell ref="I36:J36"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="I37:J37"/>
+    <mergeCell ref="K37:M37"/>
+    <mergeCell ref="G37:H37"/>
+    <mergeCell ref="J44:M44"/>
+    <mergeCell ref="F45:M45"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="F41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="J41:K41"/>
     <mergeCell ref="J54:M54"/>
     <mergeCell ref="F55:M55"/>
-    <mergeCell ref="F57:M57"/>
-    <mergeCell ref="J58:M58"/>
-    <mergeCell ref="F59:M59"/>
-    <mergeCell ref="J60:M60"/>
-    <mergeCell ref="F61:M61"/>
-    <mergeCell ref="J62:M62"/>
-    <mergeCell ref="F63:M63"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5222,6 +4765,27 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_Flow_SignoffStatus xmlns="cd6b10d8-6978-47f4-8e82-a74c94348323" xsi:nil="true"/>
+    <TaxCatchAll xmlns="38415582-292e-4658-9722-2d293e84a0eb" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cd6b10d8-6978-47f4-8e82-a74c94348323">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x010100AAE1214036CA5146B471B35D4DC55C59" ma:contentTypeVersion="17" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="a5ccbe3997558a7d0fd0136171a78fa6">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cd6b10d8-6978-47f4-8e82-a74c94348323" xmlns:ns3="38415582-292e-4658-9722-2d293e84a0eb" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6a625a2bfaeeb6abaaad9633008eb845" ns2:_="" ns3:_="">
     <xsd:import namespace="cd6b10d8-6978-47f4-8e82-a74c94348323"/>
@@ -5468,35 +5032,40 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_Flow_SignoffStatus xmlns="cd6b10d8-6978-47f4-8e82-a74c94348323" xsi:nil="true"/>
-    <TaxCatchAll xmlns="38415582-292e-4658-9722-2d293e84a0eb" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cd6b10d8-6978-47f4-8e82-a74c94348323">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB5D9902-D054-452D-A9EA-CB25CFB4B44D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4842121-BE14-4475-9250-448EBE6A0F7E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cd6b10d8-6978-47f4-8e82-a74c94348323"/>
+    <ds:schemaRef ds:uri="38415582-292e-4658-9722-2d293e84a0eb"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{130CA858-21C9-41F0-B6FE-593984D436E9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{130CA858-21C9-41F0-B6FE-593984D436E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4842121-BE14-4475-9250-448EBE6A0F7E}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BB5D9902-D054-452D-A9EA-CB25CFB4B44D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="cd6b10d8-6978-47f4-8e82-a74c94348323"/>
+    <ds:schemaRef ds:uri="38415582-292e-4658-9722-2d293e84a0eb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
regular update starting with Codex
</commit_message>
<xml_diff>
--- a/misc/regmap/sc8563_1p1_regmap.xlsx
+++ b/misc/regmap/sc8563_1p1_regmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Lab_Experiement\south_lab\misc\regmap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE2B8036-AC80-4ECA-81CB-D23A57569A9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF2CC88-1DA6-4078-A176-DC8154B3B2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="696" yWindow="2244" windowWidth="22416" windowHeight="12696" xr2:uid="{04341A28-7F9A-4CCC-96B6-6759C0F557E5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{04341A28-7F9A-4CCC-96B6-6759C0F557E5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="635" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="648" uniqueCount="403">
   <si>
     <t>0x00</t>
   </si>
@@ -1265,13 +1265,57 @@
   </si>
   <si>
     <t>DEVICE_VER[7:0]</t>
+  </si>
+  <si>
+    <t>address</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>register</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>group</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>wr</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>por</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>D7</t>
+  </si>
+  <si>
+    <t>D6</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>D4</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>D2</t>
+  </si>
+  <si>
+    <t>D1</t>
+  </si>
+  <si>
+    <t>D0</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1301,6 +1345,19 @@
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1367,7 +1424,7 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1391,6 +1448,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1727,7 +1793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3D53D8F-E1AB-4E17-A001-E0EB1C0ED563}">
-  <dimension ref="A1:M246"/>
+  <dimension ref="A1:M247"/>
   <sheetFormatPr defaultRowHeight="9.6" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="6.8984375" style="2" bestFit="1" customWidth="1"/>
@@ -1747,38 +1813,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>211</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>217</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>389</v>
-      </c>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="5"/>
-      <c r="J1" s="5"/>
-      <c r="K1" s="5"/>
-      <c r="L1" s="5"/>
-      <c r="M1" s="5"/>
+      <c r="A1" s="8" t="s">
+        <v>390</v>
+      </c>
+      <c r="B1" s="9" t="s">
+        <v>391</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>392</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>394</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>395</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>396</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>397</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>398</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>399</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>400</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>401</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="2" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>5</v>
+        <v>211</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>1</v>
@@ -1787,39 +1867,25 @@
         <v>216</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>218</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>219</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>220</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>222</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>223</v>
-      </c>
-      <c r="K2" s="1" t="s">
-        <v>224</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>225</v>
-      </c>
-      <c r="M2" s="1" t="s">
-        <v>4</v>
-      </c>
+        <v>217</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
+      <c r="I2" s="5"/>
+      <c r="J2" s="5"/>
+      <c r="K2" s="5"/>
+      <c r="L2" s="5"/>
+      <c r="M2" s="5"/>
     </row>
     <row r="3" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>1</v>
@@ -1831,36 +1897,36 @@
         <v>218</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>233</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>1</v>
@@ -1872,36 +1938,36 @@
         <v>218</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>199</v>
+        <v>229</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>200</v>
+        <v>233</v>
       </c>
     </row>
     <row r="5" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>47</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>1</v>
@@ -1913,36 +1979,36 @@
         <v>218</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>239</v>
+        <v>234</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>84</v>
+        <v>199</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>85</v>
+        <v>236</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="M5" s="1" t="s">
-        <v>243</v>
+        <v>200</v>
       </c>
     </row>
     <row r="6" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>1</v>
@@ -1954,36 +2020,36 @@
         <v>218</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>244</v>
+        <v>239</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>245</v>
+        <v>201</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>247</v>
+        <v>84</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>248</v>
+        <v>85</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
     </row>
     <row r="7" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>1</v>
@@ -1995,77 +2061,77 @@
         <v>218</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>253</v>
+        <v>245</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>254</v>
+        <v>246</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>255</v>
+        <v>247</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>256</v>
+        <v>248</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>257</v>
+        <v>249</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>202</v>
+        <v>250</v>
       </c>
       <c r="M7" s="1" t="s">
-        <v>197</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>388</v>
+        <v>216</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>258</v>
+        <v>252</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>259</v>
+        <v>253</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>260</v>
+        <v>254</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>261</v>
+        <v>255</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>86</v>
+        <v>256</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>262</v>
+        <v>257</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>263</v>
+        <v>202</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>87</v>
+        <v>197</v>
       </c>
     </row>
     <row r="9" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>1</v>
@@ -2077,36 +2143,36 @@
         <v>218</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>264</v>
+        <v>258</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>265</v>
+        <v>259</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>266</v>
+        <v>260</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>267</v>
+        <v>261</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>268</v>
+        <v>86</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="M9" s="1" t="s">
-        <v>271</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>1</v>
@@ -2118,36 +2184,36 @@
         <v>218</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>272</v>
+        <v>264</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>88</v>
+        <v>265</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>235</v>
+        <v>266</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>90</v>
+        <v>267</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>273</v>
+        <v>268</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>274</v>
+        <v>269</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>275</v>
+        <v>270</v>
       </c>
       <c r="M10" s="1" t="s">
-        <v>91</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>1</v>
@@ -2159,36 +2225,36 @@
         <v>218</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>277</v>
+        <v>235</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>94</v>
+        <v>273</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="M11" s="1" t="s">
-        <v>280</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>1</v>
@@ -2200,36 +2266,36 @@
         <v>218</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>281</v>
+        <v>276</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>282</v>
+        <v>92</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>283</v>
+        <v>277</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>284</v>
+        <v>93</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>285</v>
+        <v>94</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>286</v>
+        <v>278</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>287</v>
+        <v>279</v>
       </c>
       <c r="M12" s="1" t="s">
-        <v>288</v>
+        <v>280</v>
       </c>
     </row>
     <row r="13" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>41</v>
+        <v>53</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>1</v>
@@ -2241,77 +2307,77 @@
         <v>218</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>289</v>
+        <v>281</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>290</v>
+        <v>282</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>291</v>
+        <v>283</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>292</v>
+        <v>284</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>293</v>
+        <v>285</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>294</v>
+        <v>286</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>95</v>
+        <v>287</v>
       </c>
       <c r="M13" s="1" t="s">
-        <v>89</v>
+        <v>288</v>
       </c>
     </row>
     <row r="14" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>216</v>
+        <v>388</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>235</v>
+        <v>289</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>203</v>
+        <v>293</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>299</v>
+        <v>95</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>204</v>
+        <v>89</v>
       </c>
     </row>
     <row r="15" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>42</v>
+        <v>56</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>1</v>
@@ -2323,36 +2389,36 @@
         <v>218</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>306</v>
+        <v>235</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>235</v>
+        <v>295</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>301</v>
+        <v>297</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>302</v>
+        <v>203</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>303</v>
+        <v>298</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>304</v>
+        <v>299</v>
       </c>
       <c r="M15" s="1" t="s">
-        <v>305</v>
+        <v>204</v>
       </c>
     </row>
     <row r="16" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>1</v>
@@ -2364,36 +2430,36 @@
         <v>218</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>206</v>
+        <v>235</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>235</v>
+        <v>300</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>235</v>
+        <v>301</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>309</v>
+        <v>303</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>310</v>
+        <v>304</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>207</v>
+        <v>305</v>
       </c>
     </row>
     <row r="17" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>15</v>
+        <v>59</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>60</v>
+        <v>43</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>1</v>
@@ -2405,36 +2471,36 @@
         <v>218</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="H17" s="1" t="s">
-        <v>312</v>
+        <v>235</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>96</v>
+        <v>235</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>97</v>
+        <v>308</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="L17" s="1" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
       <c r="M17" s="1" t="s">
-        <v>315</v>
+        <v>207</v>
       </c>
     </row>
     <row r="18" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>1</v>
@@ -2446,36 +2512,36 @@
         <v>218</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>317</v>
+        <v>208</v>
       </c>
       <c r="H18" s="1" t="s">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>319</v>
+        <v>96</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>320</v>
+        <v>97</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>321</v>
+        <v>313</v>
       </c>
       <c r="L18" s="1" t="s">
-        <v>322</v>
+        <v>314</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>323</v>
+        <v>315</v>
       </c>
     </row>
     <row r="19" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>1</v>
@@ -2487,71 +2553,77 @@
         <v>218</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>324</v>
+        <v>316</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>325</v>
+        <v>317</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>327</v>
+        <v>319</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>328</v>
+        <v>320</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>329</v>
+        <v>321</v>
       </c>
       <c r="L19" s="1" t="s">
-        <v>209</v>
+        <v>322</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>205</v>
+        <v>323</v>
       </c>
     </row>
     <row r="20" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>62</v>
+        <v>44</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>388</v>
+        <v>216</v>
       </c>
       <c r="E20" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>330</v>
+        <v>324</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>331</v>
-      </c>
-      <c r="H20" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="I20" s="5"/>
+        <v>325</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>327</v>
+      </c>
       <c r="J20" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="K20" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="L20" s="5"/>
-      <c r="M20" s="5"/>
+        <v>328</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="21" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>1</v>
@@ -2563,32 +2635,30 @@
         <v>218</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>104</v>
+        <v>330</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>235</v>
+        <v>331</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="I21" s="5"/>
       <c r="J21" s="1" t="s">
-        <v>98</v>
+        <v>235</v>
       </c>
       <c r="K21" s="5" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="L21" s="5"/>
-      <c r="M21" s="1" t="s">
-        <v>99</v>
-      </c>
+      <c r="M21" s="5"/>
     </row>
     <row r="22" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>1</v>
@@ -2600,28 +2670,32 @@
         <v>218</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>235</v>
+        <v>104</v>
       </c>
       <c r="G22" s="1" t="s">
         <v>235</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="I22" s="5"/>
-      <c r="J22" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="K22" s="5"/>
+      <c r="J22" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="K22" s="5" t="s">
+        <v>335</v>
+      </c>
       <c r="L22" s="5"/>
-      <c r="M22" s="5"/>
+      <c r="M22" s="1" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="23" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>1</v>
@@ -2633,34 +2707,28 @@
         <v>218</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>100</v>
+        <v>235</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>101</v>
+        <v>235</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="I23" s="5"/>
-      <c r="J23" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="K23" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="L23" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="M23" s="1" t="s">
-        <v>120</v>
-      </c>
+      <c r="J23" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
     </row>
     <row r="24" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>1</v>
@@ -2672,34 +2740,34 @@
         <v>218</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="G24" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="H24" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="I24" s="1" t="s">
-        <v>109</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="H24" s="5" t="s">
+        <v>338</v>
+      </c>
+      <c r="I24" s="5"/>
       <c r="J24" s="1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="L24" s="5" t="s">
-        <v>134</v>
-      </c>
-      <c r="M24" s="5"/>
+        <v>103</v>
+      </c>
+      <c r="L24" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="M24" s="1" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="25" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>212</v>
+        <v>46</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>1</v>
@@ -2711,32 +2779,34 @@
         <v>218</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>339</v>
+        <v>106</v>
       </c>
       <c r="G25" s="1" t="s">
-        <v>340</v>
+        <v>107</v>
       </c>
       <c r="H25" s="1" t="s">
-        <v>341</v>
+        <v>108</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>342</v>
+        <v>109</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="L25" s="5"/>
+        <v>110</v>
+      </c>
+      <c r="K25" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L25" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="M25" s="5"/>
     </row>
     <row r="26" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>1</v>
@@ -2748,32 +2818,32 @@
         <v>218</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="G26" s="1" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="H26" s="1" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>348</v>
+        <v>235</v>
       </c>
       <c r="K26" s="5" t="s">
-        <v>349</v>
+        <v>343</v>
       </c>
       <c r="L26" s="5"/>
       <c r="M26" s="5"/>
     </row>
     <row r="27" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>66</v>
+        <v>24</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>1</v>
@@ -2785,34 +2855,32 @@
         <v>218</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>350</v>
+        <v>344</v>
       </c>
       <c r="G27" s="1" t="s">
-        <v>351</v>
+        <v>345</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>235</v>
+        <v>346</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>235</v>
+        <v>347</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="K27" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="L27" s="5" t="s">
-        <v>135</v>
-      </c>
+        <v>348</v>
+      </c>
+      <c r="K27" s="5" t="s">
+        <v>349</v>
+      </c>
+      <c r="L27" s="5"/>
       <c r="M27" s="5"/>
     </row>
     <row r="28" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>65</v>
+        <v>214</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>1</v>
@@ -2823,23 +2891,35 @@
       <c r="E28" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F28" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="G28" s="5"/>
-      <c r="H28" s="5"/>
-      <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
-      <c r="K28" s="5"/>
-      <c r="L28" s="5"/>
+      <c r="F28" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="J28" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="K28" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="L28" s="5" t="s">
+        <v>135</v>
+      </c>
       <c r="M28" s="5"/>
     </row>
     <row r="29" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>1</v>
@@ -2851,7 +2931,7 @@
         <v>218</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="G29" s="5"/>
       <c r="H29" s="5"/>
@@ -2863,10 +2943,10 @@
     </row>
     <row r="30" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>1</v>
@@ -2877,12 +2957,10 @@
       <c r="E30" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F30" s="1" t="s">
-        <v>354</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>355</v>
-      </c>
+      <c r="F30" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="G30" s="5"/>
       <c r="H30" s="5"/>
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
@@ -2892,10 +2970,10 @@
     </row>
     <row r="31" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>1</v>
@@ -2907,34 +2985,24 @@
         <v>218</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="G31" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="H31" s="1" t="s">
-        <v>235</v>
-      </c>
-      <c r="I31" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="J31" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="K31" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="L31" s="5" t="s">
-        <v>136</v>
-      </c>
+        <v>354</v>
+      </c>
+      <c r="G31" s="5" t="s">
+        <v>355</v>
+      </c>
+      <c r="H31" s="5"/>
+      <c r="I31" s="5"/>
+      <c r="J31" s="5"/>
+      <c r="K31" s="5"/>
+      <c r="L31" s="5"/>
       <c r="M31" s="5"/>
     </row>
     <row r="32" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>1</v>
@@ -2945,23 +3013,35 @@
       <c r="E32" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F32" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="G32" s="5"/>
-      <c r="H32" s="5"/>
-      <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
-      <c r="K32" s="5"/>
-      <c r="L32" s="5"/>
+      <c r="F32" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="I32" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="J32" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="K32" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="L32" s="5" t="s">
+        <v>136</v>
+      </c>
       <c r="M32" s="5"/>
     </row>
     <row r="33" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>25</v>
+        <v>76</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>1</v>
@@ -2972,12 +3052,10 @@
       <c r="E33" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F33" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="G33" s="5" t="s">
-        <v>355</v>
-      </c>
+      <c r="F33" s="5" t="s">
+        <v>356</v>
+      </c>
+      <c r="G33" s="5"/>
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
@@ -2987,10 +3065,10 @@
     </row>
     <row r="34" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>215</v>
+        <v>75</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>1</v>
@@ -3001,31 +3079,25 @@
       <c r="E34" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F34" s="3" t="s">
-        <v>119</v>
+      <c r="F34" s="1" t="s">
+        <v>357</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
-      <c r="J34" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="K34" s="3" t="s">
-        <v>121</v>
-      </c>
-      <c r="L34" s="5" t="s">
-        <v>359</v>
-      </c>
+      <c r="J34" s="5"/>
+      <c r="K34" s="5"/>
+      <c r="L34" s="5"/>
       <c r="M34" s="5"/>
     </row>
     <row r="35" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>77</v>
+        <v>215</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>1</v>
@@ -3036,23 +3108,31 @@
       <c r="E35" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F35" s="5" t="s">
-        <v>360</v>
-      </c>
-      <c r="G35" s="5"/>
+      <c r="F35" s="3" t="s">
+        <v>119</v>
+      </c>
+      <c r="G35" s="5" t="s">
+        <v>358</v>
+      </c>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
-      <c r="K35" s="5"/>
-      <c r="L35" s="5"/>
+      <c r="J35" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K35" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="L35" s="5" t="s">
+        <v>359</v>
+      </c>
       <c r="M35" s="5"/>
     </row>
     <row r="36" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>1</v>
@@ -3063,29 +3143,23 @@
       <c r="E36" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F36" s="3" t="s">
-        <v>122</v>
-      </c>
-      <c r="G36" s="5" t="s">
-        <v>361</v>
-      </c>
+      <c r="F36" s="5" t="s">
+        <v>360</v>
+      </c>
+      <c r="G36" s="5"/>
       <c r="H36" s="5"/>
-      <c r="I36" s="5" t="s">
-        <v>362</v>
-      </c>
+      <c r="I36" s="5"/>
       <c r="J36" s="5"/>
-      <c r="K36" s="5" t="s">
-        <v>363</v>
-      </c>
+      <c r="K36" s="5"/>
       <c r="L36" s="5"/>
       <c r="M36" s="5"/>
     </row>
     <row r="37" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>1</v>
@@ -3097,28 +3171,28 @@
         <v>218</v>
       </c>
       <c r="F37" s="3" t="s">
-        <v>364</v>
+        <v>122</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="H37" s="5"/>
       <c r="I37" s="5" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
       <c r="J37" s="5"/>
       <c r="K37" s="5" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="L37" s="5"/>
       <c r="M37" s="5"/>
     </row>
     <row r="38" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>1</v>
@@ -3130,26 +3204,28 @@
         <v>218</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="G38" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>368</v>
-      </c>
-      <c r="I38" s="5"/>
+        <v>364</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>365</v>
+      </c>
+      <c r="H38" s="5"/>
+      <c r="I38" s="5" t="s">
+        <v>366</v>
+      </c>
       <c r="J38" s="5"/>
-      <c r="K38" s="5"/>
+      <c r="K38" s="5" t="s">
+        <v>367</v>
+      </c>
       <c r="L38" s="5"/>
       <c r="M38" s="5"/>
     </row>
     <row r="39" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>1</v>
@@ -3160,37 +3236,27 @@
       <c r="E39" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F39" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="G39" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="H39" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="I39" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="J39" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="K39" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="L39" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="M39" s="3" t="s">
-        <v>131</v>
-      </c>
+      <c r="F39" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>368</v>
+      </c>
+      <c r="I39" s="5"/>
+      <c r="J39" s="5"/>
+      <c r="K39" s="5"/>
+      <c r="L39" s="5"/>
+      <c r="M39" s="5"/>
     </row>
     <row r="40" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>1</v>
@@ -3201,31 +3267,37 @@
       <c r="E40" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F40" s="5" t="s">
-        <v>369</v>
-      </c>
-      <c r="G40" s="5"/>
-      <c r="H40" s="5" t="s">
-        <v>370</v>
-      </c>
-      <c r="I40" s="5"/>
-      <c r="J40" s="5" t="s">
-        <v>371</v>
-      </c>
-      <c r="K40" s="5"/>
+      <c r="F40" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="I40" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="J40" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="K40" s="3" t="s">
+        <v>129</v>
+      </c>
       <c r="L40" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="M40" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="41" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>1</v>
@@ -3237,30 +3309,30 @@
         <v>218</v>
       </c>
       <c r="F41" s="5" t="s">
-        <v>374</v>
+        <v>369</v>
       </c>
       <c r="G41" s="5"/>
       <c r="H41" s="5" t="s">
-        <v>375</v>
+        <v>370</v>
       </c>
       <c r="I41" s="5"/>
       <c r="J41" s="5" t="s">
-        <v>376</v>
+        <v>371</v>
       </c>
       <c r="K41" s="5"/>
       <c r="L41" s="3" t="s">
-        <v>372</v>
+        <v>133</v>
       </c>
       <c r="M41" s="3" t="s">
-        <v>373</v>
+        <v>132</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>171</v>
+        <v>83</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>1</v>
@@ -3271,37 +3343,31 @@
       <c r="E42" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F42" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="H42" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="I42" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J42" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="K42" s="3" t="s">
-        <v>235</v>
-      </c>
+      <c r="F42" s="5" t="s">
+        <v>374</v>
+      </c>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5" t="s">
+        <v>375</v>
+      </c>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="K42" s="5"/>
       <c r="L42" s="3" t="s">
-        <v>174</v>
+        <v>372</v>
       </c>
       <c r="M42" s="3" t="s">
-        <v>175</v>
+        <v>373</v>
       </c>
     </row>
     <row r="43" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>144</v>
+        <v>34</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>145</v>
+        <v>171</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>1</v>
@@ -3313,71 +3379,77 @@
         <v>218</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>382</v>
+        <v>171</v>
       </c>
       <c r="G43" s="3" t="s">
-        <v>383</v>
+        <v>172</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="I43" s="3" t="s">
-        <v>177</v>
+        <v>235</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>178</v>
+        <v>235</v>
       </c>
       <c r="K43" s="3" t="s">
-        <v>179</v>
+        <v>235</v>
       </c>
       <c r="L43" s="3" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="M43" s="3" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
     </row>
     <row r="44" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>1</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>143</v>
+        <v>388</v>
       </c>
       <c r="E44" s="1" t="s">
         <v>218</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>235</v>
+        <v>382</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>235</v>
+        <v>383</v>
       </c>
       <c r="H44" s="3" t="s">
-        <v>235</v>
+        <v>176</v>
       </c>
       <c r="I44" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J44" s="5" t="s">
-        <v>190</v>
-      </c>
-      <c r="K44" s="5"/>
-      <c r="L44" s="5"/>
-      <c r="M44" s="5"/>
+        <v>177</v>
+      </c>
+      <c r="J44" s="3" t="s">
+        <v>178</v>
+      </c>
+      <c r="K44" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>180</v>
+      </c>
+      <c r="M44" s="3" t="s">
+        <v>181</v>
+      </c>
     </row>
     <row r="45" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>1</v>
@@ -3388,23 +3460,31 @@
       <c r="E45" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F45" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="G45" s="5"/>
-      <c r="H45" s="5"/>
-      <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
+      <c r="F45" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G45" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H45" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I45" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J45" s="5" t="s">
+        <v>190</v>
+      </c>
       <c r="K45" s="5"/>
       <c r="L45" s="5"/>
       <c r="M45" s="5"/>
     </row>
     <row r="46" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>1</v>
@@ -3415,31 +3495,23 @@
       <c r="E46" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F46" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G46" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H46" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I46" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J46" s="5" t="s">
-        <v>191</v>
-      </c>
+      <c r="F46" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="G46" s="5"/>
+      <c r="H46" s="5"/>
+      <c r="I46" s="5"/>
+      <c r="J46" s="5"/>
       <c r="K46" s="5"/>
       <c r="L46" s="5"/>
       <c r="M46" s="5"/>
     </row>
     <row r="47" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>377</v>
+        <v>151</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>1</v>
@@ -3450,23 +3522,31 @@
       <c r="E47" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F47" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="G47" s="5"/>
-      <c r="H47" s="5"/>
-      <c r="I47" s="5"/>
-      <c r="J47" s="5"/>
+      <c r="F47" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G47" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H47" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I47" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J47" s="5" t="s">
+        <v>191</v>
+      </c>
       <c r="K47" s="5"/>
       <c r="L47" s="5"/>
       <c r="M47" s="5"/>
     </row>
     <row r="48" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>1</v>
@@ -3477,31 +3557,23 @@
       <c r="E48" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F48" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G48" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H48" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I48" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J48" s="5" t="s">
-        <v>384</v>
-      </c>
+      <c r="F48" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="G48" s="5"/>
+      <c r="H48" s="5"/>
+      <c r="I48" s="5"/>
+      <c r="J48" s="5"/>
       <c r="K48" s="5"/>
       <c r="L48" s="5"/>
       <c r="M48" s="5"/>
     </row>
     <row r="49" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>35</v>
+        <v>153</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>1</v>
@@ -3512,23 +3584,31 @@
       <c r="E49" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F49" s="5" t="s">
-        <v>385</v>
-      </c>
-      <c r="G49" s="5"/>
-      <c r="H49" s="5"/>
-      <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
+      <c r="F49" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G49" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H49" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I49" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J49" s="5" t="s">
+        <v>384</v>
+      </c>
       <c r="K49" s="5"/>
       <c r="L49" s="5"/>
       <c r="M49" s="5"/>
     </row>
     <row r="50" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>1</v>
@@ -3539,31 +3619,23 @@
       <c r="E50" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F50" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G50" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H50" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I50" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J50" s="5" t="s">
-        <v>386</v>
-      </c>
+      <c r="F50" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="G50" s="5"/>
+      <c r="H50" s="5"/>
+      <c r="I50" s="5"/>
+      <c r="J50" s="5"/>
       <c r="K50" s="5"/>
       <c r="L50" s="5"/>
       <c r="M50" s="5"/>
     </row>
     <row r="51" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>1</v>
@@ -3574,23 +3646,31 @@
       <c r="E51" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F51" s="5" t="s">
-        <v>387</v>
-      </c>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
+      <c r="F51" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G51" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H51" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I51" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J51" s="5" t="s">
+        <v>386</v>
+      </c>
       <c r="K51" s="5"/>
       <c r="L51" s="5"/>
       <c r="M51" s="5"/>
     </row>
     <row r="52" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>154</v>
+        <v>381</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>1</v>
@@ -3601,31 +3681,23 @@
       <c r="E52" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F52" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G52" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H52" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I52" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J52" s="5" t="s">
-        <v>192</v>
-      </c>
+      <c r="F52" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="G52" s="5"/>
+      <c r="H52" s="5"/>
+      <c r="I52" s="5"/>
+      <c r="J52" s="5"/>
       <c r="K52" s="5"/>
       <c r="L52" s="5"/>
       <c r="M52" s="5"/>
     </row>
     <row r="53" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>137</v>
+        <v>38</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>1</v>
@@ -3636,23 +3708,31 @@
       <c r="E53" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F53" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
+      <c r="F53" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G53" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H53" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I53" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J53" s="5" t="s">
+        <v>192</v>
+      </c>
       <c r="K53" s="5"/>
       <c r="L53" s="5"/>
       <c r="M53" s="5"/>
     </row>
     <row r="54" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>1</v>
@@ -3663,31 +3743,23 @@
       <c r="E54" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F54" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G54" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H54" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I54" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J54" s="5" t="s">
-        <v>193</v>
-      </c>
+      <c r="F54" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="G54" s="5"/>
+      <c r="H54" s="5"/>
+      <c r="I54" s="5"/>
+      <c r="J54" s="5"/>
       <c r="K54" s="5"/>
       <c r="L54" s="5"/>
       <c r="M54" s="5"/>
     </row>
     <row r="55" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>1</v>
@@ -3698,23 +3770,31 @@
       <c r="E55" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F55" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="G55" s="5"/>
-      <c r="H55" s="5"/>
-      <c r="I55" s="5"/>
-      <c r="J55" s="5"/>
+      <c r="F55" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G55" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H55" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I55" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J55" s="5" t="s">
+        <v>193</v>
+      </c>
       <c r="K55" s="5"/>
       <c r="L55" s="5"/>
       <c r="M55" s="5"/>
     </row>
     <row r="56" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="C56" s="1" t="s">
         <v>1</v>
@@ -3725,35 +3805,23 @@
       <c r="E56" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="K56" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="L56" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="M56" s="7"/>
+      <c r="F56" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="G56" s="5"/>
+      <c r="H56" s="5"/>
+      <c r="I56" s="5"/>
+      <c r="J56" s="5"/>
+      <c r="K56" s="5"/>
+      <c r="L56" s="5"/>
+      <c r="M56" s="5"/>
     </row>
     <row r="57" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>1</v>
@@ -3764,23 +3832,35 @@
       <c r="E57" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F57" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="G57" s="5"/>
-      <c r="H57" s="5"/>
-      <c r="I57" s="5"/>
-      <c r="J57" s="5"/>
-      <c r="K57" s="5"/>
-      <c r="L57" s="5"/>
-      <c r="M57" s="5"/>
+      <c r="F57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="K57" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="L57" s="6" t="s">
+        <v>210</v>
+      </c>
+      <c r="M57" s="7"/>
     </row>
     <row r="58" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>160</v>
+        <v>170</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>1</v>
@@ -3791,31 +3871,23 @@
       <c r="E58" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F58" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G58" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H58" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I58" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J58" s="5" t="s">
-        <v>195</v>
-      </c>
+      <c r="F58" s="5" t="s">
+        <v>189</v>
+      </c>
+      <c r="G58" s="5"/>
+      <c r="H58" s="5"/>
+      <c r="I58" s="5"/>
+      <c r="J58" s="5"/>
       <c r="K58" s="5"/>
       <c r="L58" s="5"/>
       <c r="M58" s="5"/>
     </row>
     <row r="59" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
-        <v>161</v>
+        <v>142</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C59" s="1" t="s">
         <v>1</v>
@@ -3826,23 +3898,31 @@
       <c r="E59" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F59" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="G59" s="5"/>
-      <c r="H59" s="5"/>
-      <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
+      <c r="F59" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G59" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H59" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I59" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J59" s="5" t="s">
+        <v>195</v>
+      </c>
       <c r="K59" s="5"/>
       <c r="L59" s="5"/>
       <c r="M59" s="5"/>
     </row>
     <row r="60" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="C60" s="1" t="s">
         <v>1</v>
@@ -3853,31 +3933,23 @@
       <c r="E60" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F60" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G60" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H60" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I60" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J60" s="5" t="s">
-        <v>194</v>
-      </c>
+      <c r="F60" s="5" t="s">
+        <v>187</v>
+      </c>
+      <c r="G60" s="5"/>
+      <c r="H60" s="5"/>
+      <c r="I60" s="5"/>
+      <c r="J60" s="5"/>
       <c r="K60" s="5"/>
       <c r="L60" s="5"/>
       <c r="M60" s="5"/>
     </row>
     <row r="61" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C61" s="1" t="s">
         <v>1</v>
@@ -3888,23 +3960,31 @@
       <c r="E61" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F61" s="5" t="s">
-        <v>186</v>
-      </c>
-      <c r="G61" s="5"/>
-      <c r="H61" s="5"/>
-      <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
+      <c r="F61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I61" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J61" s="5" t="s">
+        <v>194</v>
+      </c>
       <c r="K61" s="5"/>
       <c r="L61" s="5"/>
       <c r="M61" s="5"/>
     </row>
     <row r="62" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="C62" s="1" t="s">
         <v>1</v>
@@ -3915,31 +3995,23 @@
       <c r="E62" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F62" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="G62" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="H62" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="I62" s="3" t="s">
-        <v>235</v>
-      </c>
-      <c r="J62" s="5" t="s">
-        <v>196</v>
-      </c>
+      <c r="F62" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="G62" s="5"/>
+      <c r="H62" s="5"/>
+      <c r="I62" s="5"/>
+      <c r="J62" s="5"/>
       <c r="K62" s="5"/>
       <c r="L62" s="5"/>
       <c r="M62" s="5"/>
     </row>
     <row r="63" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C63" s="1" t="s">
         <v>1</v>
@@ -3950,18 +4022,52 @@
       <c r="E63" s="1" t="s">
         <v>218</v>
       </c>
-      <c r="F63" s="5" t="s">
-        <v>188</v>
-      </c>
-      <c r="G63" s="5"/>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
+      <c r="F63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="G63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="H63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="I63" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="J63" s="5" t="s">
+        <v>196</v>
+      </c>
       <c r="K63" s="5"/>
       <c r="L63" s="5"/>
       <c r="M63" s="5"/>
     </row>
-    <row r="64" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:13" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="D64" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F64" s="5" t="s">
+        <v>188</v>
+      </c>
+      <c r="G64" s="5"/>
+      <c r="H64" s="5"/>
+      <c r="I64" s="5"/>
+      <c r="J64" s="5"/>
+      <c r="K64" s="5"/>
+      <c r="L64" s="5"/>
+      <c r="M64" s="5"/>
+    </row>
     <row r="65" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="66" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -3971,10 +4077,7 @@
     <row r="71" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="72" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="73" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E74" s="4"/>
-      <c r="F74" s="4"/>
-    </row>
+    <row r="74" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="75" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E75" s="4"/>
       <c r="F75" s="4"/>
@@ -4162,7 +4265,6 @@
     <row r="121" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E121" s="4"/>
       <c r="F121" s="4"/>
-      <c r="G121" s="4"/>
     </row>
     <row r="122" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E122" s="4"/>
@@ -4187,6 +4289,7 @@
     <row r="126" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E126" s="4"/>
       <c r="F126" s="4"/>
+      <c r="G126" s="4"/>
     </row>
     <row r="127" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E127" s="4"/>
@@ -4195,7 +4298,6 @@
     <row r="128" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E128" s="4"/>
       <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
     </row>
     <row r="129" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E129" s="4"/>
@@ -4205,24 +4307,25 @@
     <row r="130" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E130" s="4"/>
       <c r="F130" s="4"/>
+      <c r="G130" s="4"/>
     </row>
     <row r="131" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E131" s="4"/>
       <c r="F131" s="4"/>
-      <c r="G131" s="4"/>
     </row>
     <row r="132" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E132" s="4"/>
       <c r="F132" s="4"/>
+      <c r="G132" s="4"/>
     </row>
     <row r="133" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E133" s="4"/>
       <c r="F133" s="4"/>
-      <c r="G133" s="4"/>
     </row>
     <row r="134" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E134" s="4"/>
       <c r="F134" s="4"/>
+      <c r="G134" s="4"/>
     </row>
     <row r="135" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E135" s="4"/>
@@ -4247,7 +4350,6 @@
     <row r="140" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E140" s="4"/>
       <c r="F140" s="4"/>
-      <c r="G140" s="4"/>
     </row>
     <row r="141" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E141" s="4"/>
@@ -4257,11 +4359,11 @@
     <row r="142" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E142" s="4"/>
       <c r="F142" s="4"/>
+      <c r="G142" s="4"/>
     </row>
     <row r="143" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E143" s="4"/>
       <c r="F143" s="4"/>
-      <c r="G143" s="4"/>
     </row>
     <row r="144" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E144" s="4"/>
@@ -4281,6 +4383,7 @@
     <row r="147" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E147" s="4"/>
       <c r="F147" s="4"/>
+      <c r="G147" s="4"/>
     </row>
     <row r="148" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E148" s="4"/>
@@ -4317,7 +4420,6 @@
     <row r="156" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E156" s="4"/>
       <c r="F156" s="4"/>
-      <c r="G156" s="4"/>
     </row>
     <row r="157" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E157" s="4"/>
@@ -4337,6 +4439,7 @@
     <row r="160" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E160" s="4"/>
       <c r="F160" s="4"/>
+      <c r="G160" s="4"/>
     </row>
     <row r="161" spans="5:6" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E161" s="4"/>
@@ -4445,11 +4548,11 @@
     <row r="187" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E187" s="4"/>
       <c r="F187" s="4"/>
-      <c r="G187" s="4"/>
     </row>
     <row r="188" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E188" s="4"/>
       <c r="F188" s="4"/>
+      <c r="G188" s="4"/>
     </row>
     <row r="189" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E189" s="4"/>
@@ -4458,16 +4561,15 @@
     <row r="190" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E190" s="4"/>
       <c r="F190" s="4"/>
-      <c r="G190" s="4"/>
     </row>
     <row r="191" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E191" s="4"/>
       <c r="F191" s="4"/>
+      <c r="G191" s="4"/>
     </row>
     <row r="192" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E192" s="4"/>
       <c r="F192" s="4"/>
-      <c r="G192" s="4"/>
     </row>
     <row r="193" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E193" s="4"/>
@@ -4482,20 +4584,20 @@
     <row r="195" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E195" s="4"/>
       <c r="F195" s="4"/>
+      <c r="G195" s="4"/>
     </row>
     <row r="196" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E196" s="4"/>
       <c r="F196" s="4"/>
-      <c r="G196" s="4"/>
     </row>
     <row r="197" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E197" s="4"/>
       <c r="F197" s="4"/>
+      <c r="G197" s="4"/>
     </row>
     <row r="198" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E198" s="4"/>
       <c r="F198" s="4"/>
-      <c r="G198" s="4"/>
     </row>
     <row r="199" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E199" s="4"/>
@@ -4515,6 +4617,7 @@
     <row r="202" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E202" s="4"/>
       <c r="F202" s="4"/>
+      <c r="G202" s="4"/>
     </row>
     <row r="203" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E203" s="4"/>
@@ -4555,11 +4658,11 @@
     <row r="212" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E212" s="4"/>
       <c r="F212" s="4"/>
-      <c r="G212" s="4"/>
     </row>
     <row r="213" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E213" s="4"/>
       <c r="F213" s="4"/>
+      <c r="G213" s="4"/>
     </row>
     <row r="214" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E214" s="4"/>
@@ -4576,11 +4679,11 @@
     <row r="217" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E217" s="4"/>
       <c r="F217" s="4"/>
-      <c r="G217" s="4"/>
     </row>
     <row r="218" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E218" s="4"/>
       <c r="F218" s="4"/>
+      <c r="G218" s="4"/>
     </row>
     <row r="219" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E219" s="4"/>
@@ -4597,7 +4700,6 @@
     <row r="222" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E222" s="4"/>
       <c r="F222" s="4"/>
-      <c r="G222" s="4"/>
     </row>
     <row r="223" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E223" s="4"/>
@@ -4607,6 +4709,7 @@
     <row r="224" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E224" s="4"/>
       <c r="F224" s="4"/>
+      <c r="G224" s="4"/>
     </row>
     <row r="225" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E225" s="4"/>
@@ -4663,7 +4766,6 @@
     <row r="238" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E238" s="4"/>
       <c r="F238" s="4"/>
-      <c r="G238" s="4"/>
     </row>
     <row r="239" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E239" s="4"/>
@@ -4673,6 +4775,7 @@
     <row r="240" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E240" s="4"/>
       <c r="F240" s="4"/>
+      <c r="G240" s="4"/>
     </row>
     <row r="241" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E241" s="4"/>
@@ -4681,7 +4784,6 @@
     <row r="242" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E242" s="4"/>
       <c r="F242" s="4"/>
-      <c r="G242" s="4"/>
     </row>
     <row r="243" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E243" s="4"/>
@@ -4691,80 +4793,95 @@
     <row r="244" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E244" s="4"/>
       <c r="F244" s="4"/>
+      <c r="G244" s="4"/>
     </row>
     <row r="245" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E245" s="4"/>
       <c r="F245" s="4"/>
-      <c r="G245" s="4"/>
     </row>
     <row r="246" spans="5:7" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="E246" s="4"/>
       <c r="F246" s="4"/>
       <c r="G246" s="4"/>
     </row>
+    <row r="247" spans="5:7" x14ac:dyDescent="0.25">
+      <c r="E247" s="4"/>
+      <c r="F247" s="4"/>
+      <c r="G247" s="4"/>
+    </row>
   </sheetData>
   <mergeCells count="54">
-    <mergeCell ref="J62:M62"/>
-    <mergeCell ref="F63:M63"/>
-    <mergeCell ref="F57:M57"/>
-    <mergeCell ref="J58:M58"/>
-    <mergeCell ref="F59:M59"/>
-    <mergeCell ref="J60:M60"/>
-    <mergeCell ref="F61:M61"/>
-    <mergeCell ref="H38:M38"/>
-    <mergeCell ref="F51:M51"/>
-    <mergeCell ref="J52:M52"/>
-    <mergeCell ref="F53:M53"/>
-    <mergeCell ref="J46:M46"/>
-    <mergeCell ref="F47:M47"/>
-    <mergeCell ref="J48:M48"/>
-    <mergeCell ref="F49:M49"/>
-    <mergeCell ref="J50:M50"/>
-    <mergeCell ref="F40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="G33:M33"/>
-    <mergeCell ref="K25:M25"/>
-    <mergeCell ref="K26:M26"/>
-    <mergeCell ref="G34:I34"/>
-    <mergeCell ref="L34:M34"/>
-    <mergeCell ref="F28:M28"/>
-    <mergeCell ref="F29:M29"/>
-    <mergeCell ref="G30:M30"/>
-    <mergeCell ref="L31:M31"/>
-    <mergeCell ref="F32:M32"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="J22:M22"/>
-    <mergeCell ref="L24:M24"/>
-    <mergeCell ref="L27:M27"/>
-    <mergeCell ref="F1:M1"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="K20:M20"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="F35:M35"/>
-    <mergeCell ref="G36:H36"/>
-    <mergeCell ref="I36:J36"/>
-    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="L57:M57"/>
+    <mergeCell ref="J41:K41"/>
+    <mergeCell ref="F42:G42"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="J42:K42"/>
+    <mergeCell ref="J55:M55"/>
+    <mergeCell ref="F56:M56"/>
+    <mergeCell ref="F36:M36"/>
+    <mergeCell ref="G37:H37"/>
     <mergeCell ref="I37:J37"/>
     <mergeCell ref="K37:M37"/>
-    <mergeCell ref="G37:H37"/>
-    <mergeCell ref="J44:M44"/>
-    <mergeCell ref="F45:M45"/>
-    <mergeCell ref="L56:M56"/>
-    <mergeCell ref="J40:K40"/>
+    <mergeCell ref="I38:J38"/>
+    <mergeCell ref="K38:M38"/>
+    <mergeCell ref="G38:H38"/>
+    <mergeCell ref="F2:M2"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="J23:M23"/>
+    <mergeCell ref="L25:M25"/>
+    <mergeCell ref="L28:M28"/>
+    <mergeCell ref="G34:M34"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="G35:I35"/>
+    <mergeCell ref="L35:M35"/>
+    <mergeCell ref="F29:M29"/>
+    <mergeCell ref="F30:M30"/>
+    <mergeCell ref="G31:M31"/>
+    <mergeCell ref="L32:M32"/>
+    <mergeCell ref="F33:M33"/>
+    <mergeCell ref="H39:M39"/>
+    <mergeCell ref="F52:M52"/>
+    <mergeCell ref="J53:M53"/>
+    <mergeCell ref="F54:M54"/>
+    <mergeCell ref="J47:M47"/>
+    <mergeCell ref="F48:M48"/>
+    <mergeCell ref="J49:M49"/>
+    <mergeCell ref="F50:M50"/>
+    <mergeCell ref="J51:M51"/>
     <mergeCell ref="F41:G41"/>
     <mergeCell ref="H41:I41"/>
-    <mergeCell ref="J41:K41"/>
-    <mergeCell ref="J54:M54"/>
-    <mergeCell ref="F55:M55"/>
+    <mergeCell ref="J45:M45"/>
+    <mergeCell ref="F46:M46"/>
+    <mergeCell ref="J63:M63"/>
+    <mergeCell ref="F64:M64"/>
+    <mergeCell ref="F58:M58"/>
+    <mergeCell ref="J59:M59"/>
+    <mergeCell ref="F60:M60"/>
+    <mergeCell ref="J61:M61"/>
+    <mergeCell ref="F62:M62"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_Flow_SignoffStatus xmlns="cd6b10d8-6978-47f4-8e82-a74c94348323" xsi:nil="true"/>
@@ -4774,15 +4891,6 @@
     </lcf76f155ced4ddcb4097134ff3c332f>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -5033,20 +5141,20 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{130CA858-21C9-41F0-B6FE-593984D436E9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B4842121-BE14-4475-9250-448EBE6A0F7E}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="cd6b10d8-6978-47f4-8e82-a74c94348323"/>
     <ds:schemaRef ds:uri="38415582-292e-4658-9722-2d293e84a0eb"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{130CA858-21C9-41F0-B6FE-593984D436E9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>